<commit_message>
nightly Task 6+7: IE top-up scan + auto_bianche+bianche_diff+MD in one task
- data_system.py: remove standalone T5(auto_bianche) and T6(bianche_diff)
- Add T6: second-pass IE folder scan for unimported files
- Add T7: rebuild auto_bianche.xlsx → bianche_diff → update 24_DATA_SYSTEM.md
- Fix WinError 32: write auto_bianche to temp file first, then copy to final
- Update docstring to reflect tasks 0-7
- All tasks OK: T6 (0 new, 442 skip), T7 (人為差異=32)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/flask_backend/test_output/comparison_table.xlsx
+++ b/flask_backend/test_output/comparison_table.xlsx
@@ -876,21 +876,21 @@
         <v>800</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="F10" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="G10" s="4" t="n">
-        <v>17.5</v>
-      </c>
-      <c r="H10" s="4" t="n">
+      <c r="G10" s="6" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="H10" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="I10" s="4" t="n">
-        <v>21</v>
-      </c>
-      <c r="J10" s="4" t="n">
+      <c r="I10" s="6" t="n">
+        <v>39</v>
+      </c>
+      <c r="J10" s="6" t="n">
         <v>21</v>
       </c>
       <c r="K10" s="6" t="inlineStr">
@@ -1349,21 +1349,21 @@
         <v>110</v>
       </c>
       <c r="E21" s="6" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="F21" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="G21" s="4" t="n">
-        <v>17.5</v>
-      </c>
-      <c r="H21" s="4" t="n">
+      <c r="G21" s="6" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="H21" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="I21" s="4" t="n">
-        <v>21</v>
-      </c>
-      <c r="J21" s="4" t="n">
+      <c r="I21" s="6" t="n">
+        <v>39</v>
+      </c>
+      <c r="J21" s="6" t="n">
         <v>21</v>
       </c>
       <c r="K21" s="6" t="inlineStr">
@@ -1416,76 +1416,88 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>1A</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>GAZELLE GOLF</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>KJ5428</t>
         </is>
       </c>
-      <c r="D23" s="2" t="n">
+      <c r="D23" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="E23" s="2" t="n"/>
-      <c r="F23" s="2" t="n">
+      <c r="E23" s="4" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="F23" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="G23" s="2" t="n"/>
-      <c r="H23" s="2" t="n">
+      <c r="G23" s="4" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="H23" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="I23" s="2" t="n"/>
-      <c r="J23" s="2" t="n">
+      <c r="I23" s="6" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="J23" s="6" t="n">
         <v>19.5</v>
       </c>
-      <c r="K23" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K23" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>1A</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B24" s="5" t="inlineStr">
         <is>
           <t>GAZELLE GOLF</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>KJ5429</t>
         </is>
       </c>
-      <c r="D24" s="2" t="n">
+      <c r="D24" s="4" t="n">
         <v>25</v>
       </c>
-      <c r="E24" s="2" t="n"/>
-      <c r="F24" s="2" t="n">
+      <c r="E24" s="4" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="F24" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="G24" s="2" t="n"/>
-      <c r="H24" s="2" t="n">
+      <c r="G24" s="4" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="H24" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="I24" s="2" t="n"/>
-      <c r="J24" s="2" t="n">
+      <c r="I24" s="6" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="J24" s="6" t="n">
         <v>19.5</v>
       </c>
-      <c r="K24" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K24" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
@@ -2037,39 +2049,45 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="inlineStr">
+      <c r="A38" s="4" t="inlineStr">
         <is>
           <t>1C</t>
         </is>
       </c>
-      <c r="B38" s="3" t="inlineStr">
+      <c r="B38" s="5" t="inlineStr">
         <is>
           <t>R2C BOA</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr">
+      <c r="C38" s="4" t="inlineStr">
         <is>
           <t>JQ1023</t>
         </is>
       </c>
-      <c r="D38" s="2" t="n">
+      <c r="D38" s="4" t="n">
         <v>300</v>
       </c>
-      <c r="E38" s="2" t="n"/>
-      <c r="F38" s="2" t="n">
+      <c r="E38" s="6" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="F38" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="G38" s="2" t="n"/>
-      <c r="H38" s="2" t="n">
+      <c r="G38" s="4" t="n">
         <v>54</v>
       </c>
-      <c r="I38" s="2" t="n"/>
-      <c r="J38" s="2" t="n">
+      <c r="H38" s="4" t="n">
+        <v>54</v>
+      </c>
+      <c r="I38" s="4" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="J38" s="4" t="n">
         <v>35</v>
       </c>
-      <c r="K38" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K38" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
@@ -2523,39 +2541,45 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="inlineStr">
+      <c r="A50" s="4" t="inlineStr">
         <is>
           <t>2A</t>
         </is>
       </c>
-      <c r="B50" s="3" t="inlineStr">
+      <c r="B50" s="5" t="inlineStr">
         <is>
           <t>MEGARIDE F50</t>
         </is>
       </c>
-      <c r="C50" s="2" t="inlineStr">
+      <c r="C50" s="4" t="inlineStr">
         <is>
           <t>KI4715</t>
         </is>
       </c>
-      <c r="D50" s="2" t="n">
+      <c r="D50" s="4" t="n">
         <v>971</v>
       </c>
-      <c r="E50" s="2" t="n"/>
-      <c r="F50" s="2" t="n">
+      <c r="E50" s="4" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="F50" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="G50" s="2" t="n"/>
-      <c r="H50" s="2" t="n">
+      <c r="G50" s="6" t="n">
+        <v>48</v>
+      </c>
+      <c r="H50" s="6" t="n">
         <v>49</v>
       </c>
-      <c r="I50" s="2" t="n"/>
-      <c r="J50" s="2" t="n">
+      <c r="I50" s="4" t="n">
+        <v>73.5</v>
+      </c>
+      <c r="J50" s="4" t="n">
         <v>74</v>
       </c>
-      <c r="K50" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K50" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
@@ -2603,39 +2627,45 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="inlineStr">
+      <c r="A52" s="4" t="inlineStr">
         <is>
           <t>2A</t>
         </is>
       </c>
-      <c r="B52" s="3" t="inlineStr">
+      <c r="B52" s="5" t="inlineStr">
         <is>
           <t>MEGARIDE F50</t>
         </is>
       </c>
-      <c r="C52" s="2" t="inlineStr">
+      <c r="C52" s="4" t="inlineStr">
         <is>
           <t>KI4719</t>
         </is>
       </c>
-      <c r="D52" s="2" t="n">
+      <c r="D52" s="4" t="n">
         <v>287</v>
       </c>
-      <c r="E52" s="2" t="n"/>
-      <c r="F52" s="2" t="n">
+      <c r="E52" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="F52" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="G52" s="2" t="n"/>
-      <c r="H52" s="2" t="n">
+      <c r="G52" s="6" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="H52" s="6" t="n">
         <v>49</v>
       </c>
-      <c r="I52" s="2" t="n"/>
-      <c r="J52" s="2" t="n">
+      <c r="I52" s="6" t="n">
+        <v>70.5</v>
+      </c>
+      <c r="J52" s="6" t="n">
         <v>74</v>
       </c>
-      <c r="K52" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K52" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
@@ -3046,19 +3076,19 @@
         <v>598</v>
       </c>
       <c r="E62" s="6" t="n">
-        <v>13</v>
+        <v>6.5</v>
       </c>
       <c r="F62" s="6" t="n">
         <v>20</v>
       </c>
       <c r="G62" s="6" t="n">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="H62" s="6" t="n">
         <v>31</v>
       </c>
       <c r="I62" s="6" t="n">
-        <v>39.5</v>
+        <v>21.5</v>
       </c>
       <c r="J62" s="6" t="n">
         <v>41</v>
@@ -3088,20 +3118,20 @@
       <c r="D63" s="4" t="n">
         <v>221</v>
       </c>
-      <c r="E63" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="F63" s="6" t="n">
+      <c r="E63" s="4" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="F63" s="4" t="n">
         <v>20</v>
       </c>
       <c r="G63" s="6" t="n">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="H63" s="6" t="n">
         <v>31</v>
       </c>
       <c r="I63" s="6" t="n">
-        <v>20.5</v>
+        <v>36.5</v>
       </c>
       <c r="J63" s="6" t="n">
         <v>41</v>
@@ -3199,39 +3229,45 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="inlineStr">
+      <c r="A66" s="4" t="inlineStr">
         <is>
           <t>2B</t>
         </is>
       </c>
-      <c r="B66" s="3" t="inlineStr">
+      <c r="B66" s="5" t="inlineStr">
         <is>
           <t>TOKYO W</t>
         </is>
       </c>
-      <c r="C66" s="2" t="inlineStr">
+      <c r="C66" s="4" t="inlineStr">
         <is>
           <t>JI0183</t>
         </is>
       </c>
-      <c r="D66" s="2" t="n">
+      <c r="D66" s="4" t="n">
         <v>1039</v>
       </c>
-      <c r="E66" s="2" t="n"/>
-      <c r="F66" s="2" t="n">
+      <c r="E66" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="F66" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="G66" s="2" t="n"/>
-      <c r="H66" s="2" t="n">
+      <c r="G66" s="6" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="H66" s="6" t="n">
         <v>31</v>
       </c>
-      <c r="I66" s="2" t="n"/>
-      <c r="J66" s="2" t="n">
+      <c r="I66" s="6" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="J66" s="6" t="n">
         <v>41</v>
       </c>
-      <c r="K66" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K66" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
@@ -3555,20 +3591,20 @@
       <c r="D74" s="4" t="n">
         <v>3000</v>
       </c>
-      <c r="E74" s="4" t="n">
-        <v>20.5</v>
-      </c>
-      <c r="F74" s="4" t="n">
+      <c r="E74" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="F74" s="6" t="n">
         <v>20</v>
       </c>
       <c r="G74" s="6" t="n">
-        <v>32</v>
+        <v>17.5</v>
       </c>
       <c r="H74" s="6" t="n">
         <v>31</v>
       </c>
       <c r="I74" s="6" t="n">
-        <v>36.5</v>
+        <v>20.5</v>
       </c>
       <c r="J74" s="6" t="n">
         <v>41</v>
@@ -3709,39 +3745,45 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="2" t="inlineStr">
+      <c r="A78" s="4" t="inlineStr">
         <is>
           <t>2B</t>
         </is>
       </c>
-      <c r="B78" s="3" t="inlineStr">
+      <c r="B78" s="5" t="inlineStr">
         <is>
           <t>TOKYO W</t>
         </is>
       </c>
-      <c r="C78" s="2" t="inlineStr">
+      <c r="C78" s="4" t="inlineStr">
         <is>
           <t>KJ7542</t>
         </is>
       </c>
-      <c r="D78" s="2" t="n">
+      <c r="D78" s="4" t="n">
         <v>240</v>
       </c>
-      <c r="E78" s="2" t="n"/>
-      <c r="F78" s="2" t="n">
+      <c r="E78" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="G78" s="2" t="n"/>
-      <c r="H78" s="2" t="n">
+      <c r="F78" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="G78" s="4" t="n">
+        <v>31.5</v>
+      </c>
+      <c r="H78" s="4" t="n">
         <v>31</v>
       </c>
-      <c r="I78" s="2" t="n"/>
-      <c r="J78" s="2" t="n">
+      <c r="I78" s="6" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="J78" s="6" t="n">
         <v>41</v>
       </c>
-      <c r="K78" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K78" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
@@ -3789,39 +3831,45 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="2" t="inlineStr">
+      <c r="A80" s="4" t="inlineStr">
         <is>
           <t>2B</t>
         </is>
       </c>
-      <c r="B80" s="3" t="inlineStr">
+      <c r="B80" s="5" t="inlineStr">
         <is>
           <t>TOKYO W</t>
         </is>
       </c>
-      <c r="C80" s="2" t="inlineStr">
+      <c r="C80" s="4" t="inlineStr">
         <is>
           <t>KJ7544</t>
         </is>
       </c>
-      <c r="D80" s="2" t="n">
+      <c r="D80" s="4" t="n">
         <v>1310</v>
       </c>
-      <c r="E80" s="2" t="n"/>
-      <c r="F80" s="2" t="n">
+      <c r="E80" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="F80" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="G80" s="2" t="n"/>
-      <c r="H80" s="2" t="n">
+      <c r="G80" s="4" t="n">
         <v>31</v>
       </c>
-      <c r="I80" s="2" t="n"/>
-      <c r="J80" s="2" t="n">
+      <c r="H80" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="I80" s="6" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="J80" s="6" t="n">
         <v>41</v>
       </c>
-      <c r="K80" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K80" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
@@ -3845,21 +3893,21 @@
         <v>487</v>
       </c>
       <c r="E81" s="6" t="n">
-        <v>21.5</v>
+        <v>10.5</v>
       </c>
       <c r="F81" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="G81" s="4" t="n">
+      <c r="G81" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="H81" s="6" t="n">
         <v>31</v>
       </c>
-      <c r="H81" s="4" t="n">
-        <v>31</v>
-      </c>
-      <c r="I81" s="4" t="n">
-        <v>40.5</v>
-      </c>
-      <c r="J81" s="4" t="n">
+      <c r="I81" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="J81" s="6" t="n">
         <v>41</v>
       </c>
       <c r="K81" s="6" t="inlineStr">
@@ -3912,39 +3960,45 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="2" t="inlineStr">
+      <c r="A83" s="4" t="inlineStr">
         <is>
           <t>2B</t>
         </is>
       </c>
-      <c r="B83" s="3" t="inlineStr">
+      <c r="B83" s="5" t="inlineStr">
         <is>
           <t>TOKYO W</t>
         </is>
       </c>
-      <c r="C83" s="2" t="inlineStr">
+      <c r="C83" s="4" t="inlineStr">
         <is>
           <t>KK0031</t>
         </is>
       </c>
-      <c r="D83" s="2" t="n">
+      <c r="D83" s="4" t="n">
         <v>346</v>
       </c>
-      <c r="E83" s="2" t="n"/>
-      <c r="F83" s="2" t="n">
+      <c r="E83" s="6" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="F83" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="G83" s="2" t="n"/>
-      <c r="H83" s="2" t="n">
+      <c r="G83" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="H83" s="6" t="n">
         <v>31</v>
       </c>
-      <c r="I83" s="2" t="n"/>
-      <c r="J83" s="2" t="n">
+      <c r="I83" s="6" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="J83" s="6" t="n">
         <v>41</v>
       </c>
-      <c r="K83" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K83" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
@@ -3992,39 +4046,45 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="2" t="inlineStr">
+      <c r="A85" s="4" t="inlineStr">
         <is>
           <t>2B</t>
         </is>
       </c>
-      <c r="B85" s="3" t="inlineStr">
+      <c r="B85" s="5" t="inlineStr">
         <is>
           <t>TOKYO W</t>
         </is>
       </c>
-      <c r="C85" s="2" t="inlineStr">
+      <c r="C85" s="4" t="inlineStr">
         <is>
           <t>KK0037</t>
         </is>
       </c>
-      <c r="D85" s="2" t="n">
+      <c r="D85" s="4" t="n">
         <v>1638</v>
       </c>
-      <c r="E85" s="2" t="n"/>
-      <c r="F85" s="2" t="n">
+      <c r="E85" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="F85" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="G85" s="2" t="n"/>
-      <c r="H85" s="2" t="n">
+      <c r="G85" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="H85" s="6" t="n">
         <v>31</v>
       </c>
-      <c r="I85" s="2" t="n"/>
-      <c r="J85" s="2" t="n">
+      <c r="I85" s="6" t="n">
+        <v>36.5</v>
+      </c>
+      <c r="J85" s="6" t="n">
         <v>41</v>
       </c>
-      <c r="K85" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K85" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
@@ -4115,39 +4175,45 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="2" t="inlineStr">
+      <c r="A88" s="4" t="inlineStr">
         <is>
           <t>2B</t>
         </is>
       </c>
-      <c r="B88" s="3" t="inlineStr">
+      <c r="B88" s="5" t="inlineStr">
         <is>
           <t>TOKYO W</t>
         </is>
       </c>
-      <c r="C88" s="2" t="inlineStr">
+      <c r="C88" s="4" t="inlineStr">
         <is>
           <t>LA3433</t>
         </is>
       </c>
-      <c r="D88" s="2" t="n">
+      <c r="D88" s="4" t="n">
         <v>2555</v>
       </c>
-      <c r="E88" s="2" t="n"/>
-      <c r="F88" s="2" t="n">
+      <c r="E88" s="6" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="F88" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="G88" s="2" t="n"/>
-      <c r="H88" s="2" t="n">
+      <c r="G88" s="6" t="n">
+        <v>34</v>
+      </c>
+      <c r="H88" s="6" t="n">
         <v>31</v>
       </c>
-      <c r="I88" s="2" t="n"/>
-      <c r="J88" s="2" t="n">
+      <c r="I88" s="4" t="n">
+        <v>40.5</v>
+      </c>
+      <c r="J88" s="4" t="n">
         <v>41</v>
       </c>
-      <c r="K88" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K88" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
@@ -4195,39 +4261,45 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="2" t="inlineStr">
+      <c r="A90" s="4" t="inlineStr">
         <is>
           <t>2C</t>
         </is>
       </c>
-      <c r="B90" s="3" t="inlineStr">
+      <c r="B90" s="5" t="inlineStr">
         <is>
           <t>TECH RESPONSE 3.0 WD</t>
         </is>
       </c>
-      <c r="C90" s="2" t="inlineStr">
+      <c r="C90" s="4" t="inlineStr">
         <is>
           <t>GV6891</t>
         </is>
       </c>
-      <c r="D90" s="2" t="n">
+      <c r="D90" s="4" t="n">
         <v>480</v>
       </c>
-      <c r="E90" s="2" t="n"/>
-      <c r="F90" s="2" t="n">
+      <c r="E90" s="6" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="F90" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="G90" s="2" t="n"/>
-      <c r="H90" s="2" t="n">
+      <c r="G90" s="4" t="n">
         <v>34</v>
       </c>
-      <c r="I90" s="2" t="n"/>
-      <c r="J90" s="2" t="n">
+      <c r="H90" s="4" t="n">
+        <v>34</v>
+      </c>
+      <c r="I90" s="4" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="J90" s="4" t="n">
         <v>39</v>
       </c>
-      <c r="K90" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K90" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
@@ -4423,39 +4495,45 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="2" t="inlineStr">
+      <c r="A96" s="4" t="inlineStr">
         <is>
           <t>2C</t>
         </is>
       </c>
-      <c r="B96" s="3" t="inlineStr">
+      <c r="B96" s="5" t="inlineStr">
         <is>
           <t>W TECH RESPONSE 3.0</t>
         </is>
       </c>
-      <c r="C96" s="2" t="inlineStr">
+      <c r="C96" s="4" t="inlineStr">
         <is>
           <t>HQ1198</t>
         </is>
       </c>
-      <c r="D96" s="2" t="n">
+      <c r="D96" s="4" t="n">
         <v>325</v>
       </c>
-      <c r="E96" s="2" t="n"/>
-      <c r="F96" s="2" t="n">
+      <c r="E96" s="6" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="F96" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="G96" s="2" t="n"/>
-      <c r="H96" s="2" t="n">
+      <c r="G96" s="6" t="n">
+        <v>34</v>
+      </c>
+      <c r="H96" s="6" t="n">
         <v>33</v>
       </c>
-      <c r="I96" s="2" t="n"/>
-      <c r="J96" s="2" t="n">
+      <c r="I96" s="6" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="J96" s="6" t="n">
         <v>36</v>
       </c>
-      <c r="K96" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K96" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
@@ -4540,39 +4618,45 @@
       </c>
     </row>
     <row r="99">
-      <c r="A99" s="2" t="inlineStr">
+      <c r="A99" s="4" t="inlineStr">
         <is>
           <t>2C</t>
         </is>
       </c>
-      <c r="B99" s="3" t="inlineStr">
+      <c r="B99" s="5" t="inlineStr">
         <is>
           <t>TRAXION RESPONSE SL</t>
         </is>
       </c>
-      <c r="C99" s="2" t="inlineStr">
+      <c r="C99" s="4" t="inlineStr">
         <is>
           <t>IH2249</t>
         </is>
       </c>
-      <c r="D99" s="2" t="n">
+      <c r="D99" s="4" t="n">
         <v>450</v>
       </c>
-      <c r="E99" s="2" t="n"/>
-      <c r="F99" s="2" t="n">
+      <c r="E99" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="F99" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="G99" s="2" t="n"/>
-      <c r="H99" s="2" t="n">
+      <c r="G99" s="4" t="n">
         <v>39</v>
       </c>
-      <c r="I99" s="2" t="n"/>
-      <c r="J99" s="2" t="n">
+      <c r="H99" s="4" t="n">
+        <v>39</v>
+      </c>
+      <c r="I99" s="4" t="n">
         <v>37</v>
       </c>
-      <c r="K99" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="J99" s="4" t="n">
+        <v>37</v>
+      </c>
+      <c r="K99" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
@@ -4995,113 +5079,131 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="2" t="inlineStr">
+      <c r="A110" s="4" t="inlineStr">
         <is>
           <t>3A</t>
         </is>
       </c>
-      <c r="B110" s="3" t="inlineStr">
+      <c r="B110" s="5" t="inlineStr">
         <is>
           <t>LA TRAINER OG</t>
         </is>
       </c>
-      <c r="C110" s="2" t="inlineStr">
+      <c r="C110" s="4" t="inlineStr">
         <is>
           <t>KH9680</t>
         </is>
       </c>
-      <c r="D110" s="2" t="n">
+      <c r="D110" s="4" t="n">
         <v>686</v>
       </c>
-      <c r="E110" s="2" t="n"/>
-      <c r="F110" s="2" t="n">
+      <c r="E110" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="F110" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="G110" s="2" t="n"/>
-      <c r="H110" s="2" t="n">
+      <c r="G110" s="4" t="n">
         <v>33</v>
       </c>
-      <c r="I110" s="2" t="n"/>
-      <c r="J110" s="2" t="n">
+      <c r="H110" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="I110" s="4" t="n">
+        <v>41.5</v>
+      </c>
+      <c r="J110" s="4" t="n">
         <v>41</v>
       </c>
-      <c r="K110" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K110" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
     <row r="111">
-      <c r="A111" s="2" t="inlineStr">
+      <c r="A111" s="4" t="inlineStr">
         <is>
           <t>3A</t>
         </is>
       </c>
-      <c r="B111" s="3" t="inlineStr">
+      <c r="B111" s="5" t="inlineStr">
         <is>
           <t>LA TRAINER OG</t>
         </is>
       </c>
-      <c r="C111" s="2" t="inlineStr">
+      <c r="C111" s="4" t="inlineStr">
         <is>
           <t>KH9681</t>
         </is>
       </c>
-      <c r="D111" s="2" t="n">
+      <c r="D111" s="4" t="n">
         <v>418</v>
       </c>
-      <c r="E111" s="2" t="n"/>
-      <c r="F111" s="2" t="n">
+      <c r="E111" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="F111" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="G111" s="2" t="n"/>
-      <c r="H111" s="2" t="n">
+      <c r="G111" s="4" t="n">
         <v>33</v>
       </c>
-      <c r="I111" s="2" t="n"/>
-      <c r="J111" s="2" t="n">
+      <c r="H111" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="I111" s="4" t="n">
+        <v>41.5</v>
+      </c>
+      <c r="J111" s="4" t="n">
         <v>41</v>
       </c>
-      <c r="K111" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K111" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="2" t="inlineStr">
+      <c r="A112" s="4" t="inlineStr">
         <is>
           <t>3A</t>
         </is>
       </c>
-      <c r="B112" s="3" t="inlineStr">
+      <c r="B112" s="5" t="inlineStr">
         <is>
           <t>LA TRAINER OG</t>
         </is>
       </c>
-      <c r="C112" s="2" t="inlineStr">
+      <c r="C112" s="4" t="inlineStr">
         <is>
           <t>KH9683</t>
         </is>
       </c>
-      <c r="D112" s="2" t="n">
+      <c r="D112" s="4" t="n">
         <v>1616</v>
       </c>
-      <c r="E112" s="2" t="n"/>
-      <c r="F112" s="2" t="n">
+      <c r="E112" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="F112" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="G112" s="2" t="n"/>
-      <c r="H112" s="2" t="n">
+      <c r="G112" s="4" t="n">
         <v>33</v>
       </c>
-      <c r="I112" s="2" t="n"/>
-      <c r="J112" s="2" t="n">
+      <c r="H112" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="I112" s="6" t="n">
+        <v>39.5</v>
+      </c>
+      <c r="J112" s="6" t="n">
         <v>41</v>
       </c>
-      <c r="K112" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K112" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
@@ -5217,76 +5319,88 @@
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="2" t="inlineStr">
+      <c r="A116" s="4" t="inlineStr">
         <is>
           <t>3A</t>
         </is>
       </c>
-      <c r="B116" s="3" t="inlineStr">
+      <c r="B116" s="5" t="inlineStr">
         <is>
           <t>LA TRAINER OG</t>
         </is>
       </c>
-      <c r="C116" s="2" t="inlineStr">
+      <c r="C116" s="4" t="inlineStr">
         <is>
           <t>KJ4381</t>
         </is>
       </c>
-      <c r="D116" s="2" t="n">
+      <c r="D116" s="4" t="n">
         <v>200</v>
       </c>
-      <c r="E116" s="2" t="n"/>
-      <c r="F116" s="2" t="n">
+      <c r="E116" s="6" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="F116" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="G116" s="2" t="n"/>
-      <c r="H116" s="2" t="n">
+      <c r="G116" s="4" t="n">
         <v>33</v>
       </c>
-      <c r="I116" s="2" t="n"/>
-      <c r="J116" s="2" t="n">
+      <c r="H116" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="I116" s="4" t="n">
+        <v>40.5</v>
+      </c>
+      <c r="J116" s="4" t="n">
         <v>41</v>
       </c>
-      <c r="K116" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K116" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="2" t="inlineStr">
+      <c r="A117" s="4" t="inlineStr">
         <is>
           <t>3A</t>
         </is>
       </c>
-      <c r="B117" s="3" t="inlineStr">
+      <c r="B117" s="5" t="inlineStr">
         <is>
           <t>LA TRAINER OG</t>
         </is>
       </c>
-      <c r="C117" s="2" t="inlineStr">
+      <c r="C117" s="4" t="inlineStr">
         <is>
           <t>KJ4382</t>
         </is>
       </c>
-      <c r="D117" s="2" t="n">
+      <c r="D117" s="4" t="n">
         <v>2903</v>
       </c>
-      <c r="E117" s="2" t="n"/>
-      <c r="F117" s="2" t="n">
+      <c r="E117" s="6" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="F117" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="G117" s="2" t="n"/>
-      <c r="H117" s="2" t="n">
+      <c r="G117" s="4" t="n">
         <v>33</v>
       </c>
-      <c r="I117" s="2" t="n"/>
-      <c r="J117" s="2" t="n">
+      <c r="H117" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="I117" s="4" t="n">
+        <v>40.5</v>
+      </c>
+      <c r="J117" s="4" t="n">
         <v>41</v>
       </c>
-      <c r="K117" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K117" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
@@ -5556,39 +5670,45 @@
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="2" t="inlineStr">
+      <c r="A125" s="4" t="inlineStr">
         <is>
           <t>3B</t>
         </is>
       </c>
-      <c r="B125" s="3" t="inlineStr">
+      <c r="B125" s="5" t="inlineStr">
         <is>
           <t>SAMBA J</t>
         </is>
       </c>
-      <c r="C125" s="2" t="inlineStr">
+      <c r="C125" s="4" t="inlineStr">
         <is>
           <t>IF1945</t>
         </is>
       </c>
-      <c r="D125" s="2" t="n">
+      <c r="D125" s="4" t="n">
         <v>1336</v>
       </c>
-      <c r="E125" s="2" t="n"/>
-      <c r="F125" s="2" t="n">
+      <c r="E125" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="F125" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="G125" s="2" t="n"/>
-      <c r="H125" s="2" t="n">
+      <c r="G125" s="6" t="n">
+        <v>32</v>
+      </c>
+      <c r="H125" s="6" t="n">
         <v>31</v>
       </c>
-      <c r="I125" s="2" t="n"/>
-      <c r="J125" s="2" t="n">
+      <c r="I125" s="6" t="n">
+        <v>38</v>
+      </c>
+      <c r="J125" s="6" t="n">
         <v>39</v>
       </c>
-      <c r="K125" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K125" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
@@ -5655,19 +5775,19 @@
         <v>2500</v>
       </c>
       <c r="E127" s="6" t="n">
-        <v>14.5</v>
+        <v>8.5</v>
       </c>
       <c r="F127" s="6" t="n">
         <v>12</v>
       </c>
       <c r="G127" s="6" t="n">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="H127" s="6" t="n">
         <v>31</v>
       </c>
       <c r="I127" s="6" t="n">
-        <v>40</v>
+        <v>22</v>
       </c>
       <c r="J127" s="6" t="n">
         <v>39</v>
@@ -6468,76 +6588,88 @@
       </c>
     </row>
     <row r="149">
-      <c r="A149" s="2" t="inlineStr">
+      <c r="A149" s="4" t="inlineStr">
         <is>
           <t>5A</t>
         </is>
       </c>
-      <c r="B149" s="3" t="inlineStr">
+      <c r="B149" s="5" t="inlineStr">
         <is>
           <t>ORGN ULTRA TECH</t>
         </is>
       </c>
-      <c r="C149" s="2" t="inlineStr">
+      <c r="C149" s="4" t="inlineStr">
         <is>
           <t>KI7557</t>
         </is>
       </c>
-      <c r="D149" s="2" t="n">
+      <c r="D149" s="4" t="n">
         <v>1500</v>
       </c>
-      <c r="E149" s="2" t="n"/>
-      <c r="F149" s="2" t="n">
+      <c r="E149" s="4" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="F149" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="G149" s="2" t="n"/>
-      <c r="H149" s="2" t="n">
+      <c r="G149" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="I149" s="2" t="n"/>
-      <c r="J149" s="2" t="n">
+      <c r="H149" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="I149" s="6" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="J149" s="6" t="n">
         <v>41</v>
       </c>
-      <c r="K149" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K149" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
     <row r="150">
-      <c r="A150" s="2" t="inlineStr">
+      <c r="A150" s="4" t="inlineStr">
         <is>
           <t>5A</t>
         </is>
       </c>
-      <c r="B150" s="3" t="inlineStr">
+      <c r="B150" s="5" t="inlineStr">
         <is>
           <t>ORGN ULTRA TECH</t>
         </is>
       </c>
-      <c r="C150" s="2" t="inlineStr">
+      <c r="C150" s="4" t="inlineStr">
         <is>
           <t>KI7558</t>
         </is>
       </c>
-      <c r="D150" s="2" t="n">
+      <c r="D150" s="4" t="n">
         <v>4250</v>
       </c>
-      <c r="E150" s="2" t="n"/>
-      <c r="F150" s="2" t="n">
+      <c r="E150" s="4" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="F150" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="G150" s="2" t="n"/>
-      <c r="H150" s="2" t="n">
+      <c r="G150" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="I150" s="2" t="n"/>
-      <c r="J150" s="2" t="n">
+      <c r="H150" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="I150" s="6" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="J150" s="6" t="n">
         <v>41</v>
       </c>
-      <c r="K150" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K150" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
@@ -6585,113 +6717,131 @@
       </c>
     </row>
     <row r="152">
-      <c r="A152" s="2" t="inlineStr">
+      <c r="A152" s="4" t="inlineStr">
         <is>
           <t>5A</t>
         </is>
       </c>
-      <c r="B152" s="3" t="inlineStr">
+      <c r="B152" s="5" t="inlineStr">
         <is>
           <t>ORGN ULTRA TECH</t>
         </is>
       </c>
-      <c r="C152" s="2" t="inlineStr">
+      <c r="C152" s="4" t="inlineStr">
         <is>
           <t>KJ5260</t>
         </is>
       </c>
-      <c r="D152" s="2" t="n">
+      <c r="D152" s="4" t="n">
         <v>1211</v>
       </c>
-      <c r="E152" s="2" t="n"/>
-      <c r="F152" s="2" t="n">
+      <c r="E152" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="F152" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="G152" s="2" t="n"/>
-      <c r="H152" s="2" t="n">
+      <c r="G152" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="I152" s="2" t="n"/>
-      <c r="J152" s="2" t="n">
+      <c r="H152" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="I152" s="6" t="n">
+        <v>39.5</v>
+      </c>
+      <c r="J152" s="6" t="n">
         <v>41</v>
       </c>
-      <c r="K152" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K152" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
     <row r="153">
-      <c r="A153" s="2" t="inlineStr">
+      <c r="A153" s="4" t="inlineStr">
         <is>
           <t>5A</t>
         </is>
       </c>
-      <c r="B153" s="3" t="inlineStr">
+      <c r="B153" s="5" t="inlineStr">
         <is>
           <t>ORGN ULTRA TECH</t>
         </is>
       </c>
-      <c r="C153" s="2" t="inlineStr">
+      <c r="C153" s="4" t="inlineStr">
         <is>
           <t>KJ5261</t>
         </is>
       </c>
-      <c r="D153" s="2" t="n">
+      <c r="D153" s="4" t="n">
         <v>504</v>
       </c>
-      <c r="E153" s="2" t="n"/>
-      <c r="F153" s="2" t="n">
+      <c r="E153" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="F153" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="G153" s="2" t="n"/>
-      <c r="H153" s="2" t="n">
+      <c r="G153" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="I153" s="2" t="n"/>
-      <c r="J153" s="2" t="n">
+      <c r="H153" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="I153" s="6" t="n">
+        <v>39.5</v>
+      </c>
+      <c r="J153" s="6" t="n">
         <v>41</v>
       </c>
-      <c r="K153" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K153" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
     <row r="154">
-      <c r="A154" s="2" t="inlineStr">
+      <c r="A154" s="4" t="inlineStr">
         <is>
           <t>5A</t>
         </is>
       </c>
-      <c r="B154" s="3" t="inlineStr">
+      <c r="B154" s="5" t="inlineStr">
         <is>
           <t>ORGN ULTRA TECH</t>
         </is>
       </c>
-      <c r="C154" s="2" t="inlineStr">
+      <c r="C154" s="4" t="inlineStr">
         <is>
           <t>KJ8322</t>
         </is>
       </c>
-      <c r="D154" s="2" t="n">
+      <c r="D154" s="4" t="n">
         <v>450</v>
       </c>
-      <c r="E154" s="2" t="n"/>
-      <c r="F154" s="2" t="n">
+      <c r="E154" s="4" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="F154" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="G154" s="2" t="n"/>
-      <c r="H154" s="2" t="n">
+      <c r="G154" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="I154" s="2" t="n"/>
-      <c r="J154" s="2" t="n">
+      <c r="H154" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="I154" s="6" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="J154" s="6" t="n">
         <v>41</v>
       </c>
-      <c r="K154" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K154" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
@@ -6739,39 +6889,45 @@
       </c>
     </row>
     <row r="156">
-      <c r="A156" s="2" t="inlineStr">
+      <c r="A156" s="4" t="inlineStr">
         <is>
           <t>5A</t>
         </is>
       </c>
-      <c r="B156" s="3" t="inlineStr">
+      <c r="B156" s="5" t="inlineStr">
         <is>
           <t>ORGN ULTRA TECH</t>
         </is>
       </c>
-      <c r="C156" s="2" t="inlineStr">
+      <c r="C156" s="4" t="inlineStr">
         <is>
           <t>KZ6382</t>
         </is>
       </c>
-      <c r="D156" s="2" t="n">
+      <c r="D156" s="4" t="n">
         <v>600</v>
       </c>
-      <c r="E156" s="2" t="n"/>
-      <c r="F156" s="2" t="n">
+      <c r="E156" s="6" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="F156" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="G156" s="2" t="n"/>
-      <c r="H156" s="2" t="n">
+      <c r="G156" s="6" t="n">
+        <v>56</v>
+      </c>
+      <c r="H156" s="6" t="n">
         <v>50</v>
       </c>
-      <c r="I156" s="2" t="n"/>
-      <c r="J156" s="2" t="n">
+      <c r="I156" s="6" t="n">
+        <v>39.5</v>
+      </c>
+      <c r="J156" s="6" t="n">
         <v>41</v>
       </c>
-      <c r="K156" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K156" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
@@ -6811,31 +6967,37 @@
       </c>
     </row>
     <row r="158">
-      <c r="A158" s="2" t="inlineStr">
+      <c r="A158" s="4" t="inlineStr">
         <is>
           <t>5C</t>
         </is>
       </c>
-      <c r="B158" s="3" t="inlineStr"/>
-      <c r="C158" s="2" t="inlineStr">
+      <c r="B158" s="5" t="inlineStr"/>
+      <c r="C158" s="4" t="inlineStr">
         <is>
           <t>HP5124</t>
         </is>
       </c>
-      <c r="D158" s="2" t="n">
+      <c r="D158" s="4" t="n">
         <v>2515</v>
       </c>
-      <c r="E158" s="2" t="n"/>
-      <c r="F158" s="2" t="n"/>
-      <c r="G158" s="2" t="n"/>
-      <c r="H158" s="2" t="n"/>
-      <c r="I158" s="2" t="n"/>
-      <c r="J158" s="2" t="n">
+      <c r="E158" s="4" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="F158" s="6" t="n"/>
+      <c r="G158" s="4" t="n">
+        <v>39.5</v>
+      </c>
+      <c r="H158" s="6" t="n"/>
+      <c r="I158" s="6" t="n">
+        <v>39.5</v>
+      </c>
+      <c r="J158" s="6" t="n">
         <v>42</v>
       </c>
-      <c r="K158" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K158" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
@@ -6951,200 +7113,236 @@
       </c>
     </row>
     <row r="162">
-      <c r="A162" s="2" t="inlineStr">
+      <c r="A162" s="4" t="inlineStr">
         <is>
           <t>5C</t>
         </is>
       </c>
-      <c r="B162" s="3" t="inlineStr">
+      <c r="B162" s="5" t="inlineStr">
         <is>
           <t>SL 72 RS</t>
         </is>
       </c>
-      <c r="C162" s="2" t="inlineStr">
+      <c r="C162" s="4" t="inlineStr">
         <is>
           <t>JQ9555</t>
         </is>
       </c>
-      <c r="D162" s="2" t="n">
+      <c r="D162" s="4" t="n">
         <v>475</v>
       </c>
-      <c r="E162" s="2" t="n"/>
-      <c r="F162" s="2" t="n"/>
-      <c r="G162" s="2" t="n"/>
-      <c r="H162" s="2" t="n"/>
-      <c r="I162" s="2" t="n"/>
-      <c r="J162" s="2" t="n">
+      <c r="E162" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="F162" s="6" t="n"/>
+      <c r="G162" s="4" t="n">
+        <v>31.5</v>
+      </c>
+      <c r="H162" s="6" t="n"/>
+      <c r="I162" s="6" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="J162" s="6" t="n">
         <v>41</v>
       </c>
-      <c r="K162" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K162" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
     <row r="163">
-      <c r="A163" s="2" t="inlineStr">
+      <c r="A163" s="4" t="inlineStr">
         <is>
           <t>5C</t>
         </is>
       </c>
-      <c r="B163" s="3" t="inlineStr">
+      <c r="B163" s="5" t="inlineStr">
         <is>
           <t>SL 72 RS</t>
         </is>
       </c>
-      <c r="C163" s="2" t="inlineStr">
+      <c r="C163" s="4" t="inlineStr">
         <is>
           <t>JQ9824</t>
         </is>
       </c>
-      <c r="D163" s="2" t="n">
+      <c r="D163" s="4" t="n">
         <v>3216</v>
       </c>
-      <c r="E163" s="2" t="n"/>
-      <c r="F163" s="2" t="n"/>
-      <c r="G163" s="2" t="n"/>
-      <c r="H163" s="2" t="n"/>
-      <c r="I163" s="2" t="n"/>
-      <c r="J163" s="2" t="n">
+      <c r="E163" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="F163" s="6" t="n"/>
+      <c r="G163" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="H163" s="6" t="n"/>
+      <c r="I163" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="J163" s="6" t="n">
         <v>41</v>
       </c>
-      <c r="K163" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K163" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
     <row r="164">
-      <c r="A164" s="2" t="inlineStr">
+      <c r="A164" s="4" t="inlineStr">
         <is>
           <t>5C</t>
         </is>
       </c>
-      <c r="B164" s="3" t="inlineStr">
+      <c r="B164" s="5" t="inlineStr">
         <is>
           <t>SL 72 RS</t>
         </is>
       </c>
-      <c r="C164" s="2" t="inlineStr">
+      <c r="C164" s="4" t="inlineStr">
         <is>
           <t>KH9644</t>
         </is>
       </c>
-      <c r="D164" s="2" t="n">
+      <c r="D164" s="4" t="n">
         <v>90</v>
       </c>
-      <c r="E164" s="2" t="n"/>
-      <c r="F164" s="2" t="n"/>
-      <c r="G164" s="2" t="n"/>
-      <c r="H164" s="2" t="n"/>
-      <c r="I164" s="2" t="n"/>
-      <c r="J164" s="2" t="n">
+      <c r="E164" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="F164" s="6" t="n"/>
+      <c r="G164" s="4" t="n">
+        <v>31.5</v>
+      </c>
+      <c r="H164" s="6" t="n"/>
+      <c r="I164" s="6" t="n">
+        <v>39</v>
+      </c>
+      <c r="J164" s="6" t="n">
         <v>41</v>
       </c>
-      <c r="K164" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K164" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
     <row r="165">
-      <c r="A165" s="2" t="inlineStr">
+      <c r="A165" s="4" t="inlineStr">
         <is>
           <t>5C</t>
         </is>
       </c>
-      <c r="B165" s="3" t="inlineStr">
+      <c r="B165" s="5" t="inlineStr">
         <is>
           <t>SL 72 RS</t>
         </is>
       </c>
-      <c r="C165" s="2" t="inlineStr">
+      <c r="C165" s="4" t="inlineStr">
         <is>
           <t>KH9646</t>
         </is>
       </c>
-      <c r="D165" s="2" t="n">
+      <c r="D165" s="4" t="n">
         <v>673</v>
       </c>
-      <c r="E165" s="2" t="n"/>
-      <c r="F165" s="2" t="n"/>
-      <c r="G165" s="2" t="n"/>
-      <c r="H165" s="2" t="n"/>
-      <c r="I165" s="2" t="n"/>
-      <c r="J165" s="2" t="n">
+      <c r="E165" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="F165" s="6" t="n"/>
+      <c r="G165" s="4" t="n">
+        <v>31.5</v>
+      </c>
+      <c r="H165" s="6" t="n"/>
+      <c r="I165" s="6" t="n">
+        <v>39</v>
+      </c>
+      <c r="J165" s="6" t="n">
         <v>41</v>
       </c>
-      <c r="K165" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K165" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
     <row r="166">
-      <c r="A166" s="2" t="inlineStr">
+      <c r="A166" s="4" t="inlineStr">
         <is>
           <t>5C</t>
         </is>
       </c>
-      <c r="B166" s="3" t="inlineStr">
+      <c r="B166" s="5" t="inlineStr">
         <is>
           <t>SL 72 RS</t>
         </is>
       </c>
-      <c r="C166" s="2" t="inlineStr">
+      <c r="C166" s="4" t="inlineStr">
         <is>
           <t>KH9647</t>
         </is>
       </c>
-      <c r="D166" s="2" t="n">
+      <c r="D166" s="4" t="n">
         <v>155</v>
       </c>
-      <c r="E166" s="2" t="n"/>
-      <c r="F166" s="2" t="n"/>
-      <c r="G166" s="2" t="n"/>
-      <c r="H166" s="2" t="n"/>
-      <c r="I166" s="2" t="n"/>
-      <c r="J166" s="2" t="n">
+      <c r="E166" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="F166" s="6" t="n"/>
+      <c r="G166" s="4" t="n">
+        <v>31.5</v>
+      </c>
+      <c r="H166" s="6" t="n"/>
+      <c r="I166" s="6" t="n">
+        <v>39</v>
+      </c>
+      <c r="J166" s="6" t="n">
         <v>41</v>
       </c>
-      <c r="K166" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K166" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
     <row r="167">
-      <c r="A167" s="2" t="inlineStr">
+      <c r="A167" s="4" t="inlineStr">
         <is>
           <t>5C</t>
         </is>
       </c>
-      <c r="B167" s="3" t="inlineStr">
+      <c r="B167" s="5" t="inlineStr">
         <is>
           <t>SL 72 RS</t>
         </is>
       </c>
-      <c r="C167" s="2" t="inlineStr">
+      <c r="C167" s="4" t="inlineStr">
         <is>
           <t>KH9648</t>
         </is>
       </c>
-      <c r="D167" s="2" t="n">
+      <c r="D167" s="4" t="n">
         <v>1104</v>
       </c>
-      <c r="E167" s="2" t="n"/>
-      <c r="F167" s="2" t="n"/>
-      <c r="G167" s="2" t="n"/>
-      <c r="H167" s="2" t="n"/>
-      <c r="I167" s="2" t="n"/>
-      <c r="J167" s="2" t="n">
+      <c r="E167" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="F167" s="6" t="n"/>
+      <c r="G167" s="4" t="n">
+        <v>31.5</v>
+      </c>
+      <c r="H167" s="6" t="n"/>
+      <c r="I167" s="6" t="n">
+        <v>39</v>
+      </c>
+      <c r="J167" s="6" t="n">
         <v>41</v>
       </c>
-      <c r="K167" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K167" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
@@ -7221,134 +7419,158 @@
       </c>
     </row>
     <row r="170">
-      <c r="A170" s="2" t="inlineStr">
+      <c r="A170" s="4" t="inlineStr">
         <is>
           <t>5C</t>
         </is>
       </c>
-      <c r="B170" s="3" t="inlineStr">
+      <c r="B170" s="5" t="inlineStr">
         <is>
           <t>SL 72 RS</t>
         </is>
       </c>
-      <c r="C170" s="2" t="inlineStr">
+      <c r="C170" s="4" t="inlineStr">
         <is>
           <t>KH9652</t>
         </is>
       </c>
-      <c r="D170" s="2" t="n">
+      <c r="D170" s="4" t="n">
         <v>770</v>
       </c>
-      <c r="E170" s="2" t="n"/>
-      <c r="F170" s="2" t="n"/>
-      <c r="G170" s="2" t="n"/>
-      <c r="H170" s="2" t="n"/>
-      <c r="I170" s="2" t="n"/>
-      <c r="J170" s="2" t="n">
+      <c r="E170" s="4" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="F170" s="6" t="n"/>
+      <c r="G170" s="4" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="H170" s="6" t="n"/>
+      <c r="I170" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="J170" s="6" t="n">
         <v>41</v>
       </c>
-      <c r="K170" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K170" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
     <row r="171">
-      <c r="A171" s="2" t="inlineStr">
+      <c r="A171" s="4" t="inlineStr">
         <is>
           <t>5C</t>
         </is>
       </c>
-      <c r="B171" s="3" t="inlineStr">
+      <c r="B171" s="5" t="inlineStr">
         <is>
           <t>SL 72 RS</t>
         </is>
       </c>
-      <c r="C171" s="2" t="inlineStr">
+      <c r="C171" s="4" t="inlineStr">
         <is>
           <t>KH9653</t>
         </is>
       </c>
-      <c r="D171" s="2" t="n">
+      <c r="D171" s="4" t="n">
         <v>1442</v>
       </c>
-      <c r="E171" s="2" t="n"/>
-      <c r="F171" s="2" t="n"/>
-      <c r="G171" s="2" t="n"/>
-      <c r="H171" s="2" t="n"/>
-      <c r="I171" s="2" t="n"/>
-      <c r="J171" s="2" t="n">
+      <c r="E171" s="4" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="F171" s="6" t="n"/>
+      <c r="G171" s="4" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="H171" s="6" t="n"/>
+      <c r="I171" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="J171" s="6" t="n">
         <v>41</v>
       </c>
-      <c r="K171" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K171" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
     <row r="172">
-      <c r="A172" s="2" t="inlineStr">
+      <c r="A172" s="4" t="inlineStr">
         <is>
           <t>5C</t>
         </is>
       </c>
-      <c r="B172" s="3" t="inlineStr">
+      <c r="B172" s="5" t="inlineStr">
         <is>
           <t>SL 72 RS</t>
         </is>
       </c>
-      <c r="C172" s="2" t="inlineStr">
+      <c r="C172" s="4" t="inlineStr">
         <is>
           <t>KH9656</t>
         </is>
       </c>
-      <c r="D172" s="2" t="n">
+      <c r="D172" s="4" t="n">
         <v>152</v>
       </c>
-      <c r="E172" s="2" t="n"/>
-      <c r="F172" s="2" t="n"/>
-      <c r="G172" s="2" t="n"/>
-      <c r="H172" s="2" t="n"/>
-      <c r="I172" s="2" t="n"/>
-      <c r="J172" s="2" t="n">
+      <c r="E172" s="4" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="F172" s="6" t="n"/>
+      <c r="G172" s="4" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="H172" s="6" t="n"/>
+      <c r="I172" s="6" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="J172" s="6" t="n">
         <v>41</v>
       </c>
-      <c r="K172" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K172" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
     <row r="173">
-      <c r="A173" s="2" t="inlineStr">
+      <c r="A173" s="4" t="inlineStr">
         <is>
           <t>5C</t>
         </is>
       </c>
-      <c r="B173" s="3" t="inlineStr">
+      <c r="B173" s="5" t="inlineStr">
         <is>
           <t>SL 72 RS</t>
         </is>
       </c>
-      <c r="C173" s="2" t="inlineStr">
+      <c r="C173" s="4" t="inlineStr">
         <is>
           <t>KH9657</t>
         </is>
       </c>
-      <c r="D173" s="2" t="n">
+      <c r="D173" s="4" t="n">
         <v>300</v>
       </c>
-      <c r="E173" s="2" t="n"/>
-      <c r="F173" s="2" t="n"/>
-      <c r="G173" s="2" t="n"/>
-      <c r="H173" s="2" t="n"/>
-      <c r="I173" s="2" t="n"/>
-      <c r="J173" s="2" t="n">
+      <c r="E173" s="4" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="F173" s="6" t="n"/>
+      <c r="G173" s="4" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="H173" s="6" t="n"/>
+      <c r="I173" s="6" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="J173" s="6" t="n">
         <v>41</v>
       </c>
-      <c r="K173" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K173" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
@@ -7431,68 +7653,80 @@
       </c>
     </row>
     <row r="176">
-      <c r="A176" s="2" t="inlineStr">
+      <c r="A176" s="4" t="inlineStr">
         <is>
           <t>5C</t>
         </is>
       </c>
-      <c r="B176" s="3" t="inlineStr">
+      <c r="B176" s="5" t="inlineStr">
         <is>
           <t>SL 72 RS</t>
         </is>
       </c>
-      <c r="C176" s="2" t="inlineStr">
+      <c r="C176" s="4" t="inlineStr">
         <is>
           <t>KH9672</t>
         </is>
       </c>
-      <c r="D176" s="2" t="n">
+      <c r="D176" s="4" t="n">
         <v>771</v>
       </c>
-      <c r="E176" s="2" t="n"/>
-      <c r="F176" s="2" t="n"/>
-      <c r="G176" s="2" t="n"/>
-      <c r="H176" s="2" t="n"/>
-      <c r="I176" s="2" t="n"/>
-      <c r="J176" s="2" t="n">
+      <c r="E176" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="F176" s="6" t="n"/>
+      <c r="G176" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="H176" s="6" t="n"/>
+      <c r="I176" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="J176" s="6" t="n">
         <v>41</v>
       </c>
-      <c r="K176" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K176" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
     <row r="177">
-      <c r="A177" s="2" t="inlineStr">
+      <c r="A177" s="4" t="inlineStr">
         <is>
           <t>5C</t>
         </is>
       </c>
-      <c r="B177" s="3" t="inlineStr">
+      <c r="B177" s="5" t="inlineStr">
         <is>
           <t>SL 72 RS</t>
         </is>
       </c>
-      <c r="C177" s="2" t="inlineStr">
+      <c r="C177" s="4" t="inlineStr">
         <is>
           <t>KH9673</t>
         </is>
       </c>
-      <c r="D177" s="2" t="n">
+      <c r="D177" s="4" t="n">
         <v>2488</v>
       </c>
-      <c r="E177" s="2" t="n"/>
-      <c r="F177" s="2" t="n"/>
-      <c r="G177" s="2" t="n"/>
-      <c r="H177" s="2" t="n"/>
-      <c r="I177" s="2" t="n"/>
-      <c r="J177" s="2" t="n">
+      <c r="E177" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="F177" s="6" t="n"/>
+      <c r="G177" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="H177" s="6" t="n"/>
+      <c r="I177" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="J177" s="6" t="n">
         <v>41</v>
       </c>
-      <c r="K177" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K177" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
@@ -7575,35 +7809,41 @@
       </c>
     </row>
     <row r="180">
-      <c r="A180" s="2" t="inlineStr">
+      <c r="A180" s="4" t="inlineStr">
         <is>
           <t>5C</t>
         </is>
       </c>
-      <c r="B180" s="3" t="inlineStr">
+      <c r="B180" s="5" t="inlineStr">
         <is>
           <t>SL 72 RS</t>
         </is>
       </c>
-      <c r="C180" s="2" t="inlineStr">
+      <c r="C180" s="4" t="inlineStr">
         <is>
           <t>KJ1667</t>
         </is>
       </c>
-      <c r="D180" s="2" t="n">
+      <c r="D180" s="4" t="n">
         <v>1700</v>
       </c>
-      <c r="E180" s="2" t="n"/>
-      <c r="F180" s="2" t="n"/>
-      <c r="G180" s="2" t="n"/>
-      <c r="H180" s="2" t="n"/>
-      <c r="I180" s="2" t="n"/>
-      <c r="J180" s="2" t="n">
+      <c r="E180" s="4" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="F180" s="6" t="n"/>
+      <c r="G180" s="4" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="H180" s="6" t="n"/>
+      <c r="I180" s="6" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="J180" s="6" t="n">
         <v>41</v>
       </c>
-      <c r="K180" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K180" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
@@ -7647,101 +7887,119 @@
       </c>
     </row>
     <row r="182">
-      <c r="A182" s="2" t="inlineStr">
+      <c r="A182" s="4" t="inlineStr">
         <is>
           <t>5C</t>
         </is>
       </c>
-      <c r="B182" s="3" t="inlineStr">
+      <c r="B182" s="5" t="inlineStr">
         <is>
           <t>SL 72 RS</t>
         </is>
       </c>
-      <c r="C182" s="2" t="inlineStr">
+      <c r="C182" s="4" t="inlineStr">
         <is>
           <t>KJ1670</t>
         </is>
       </c>
-      <c r="D182" s="2" t="n">
+      <c r="D182" s="4" t="n">
         <v>1256</v>
       </c>
-      <c r="E182" s="2" t="n"/>
-      <c r="F182" s="2" t="n"/>
-      <c r="G182" s="2" t="n"/>
-      <c r="H182" s="2" t="n"/>
-      <c r="I182" s="2" t="n"/>
-      <c r="J182" s="2" t="n">
+      <c r="E182" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="F182" s="6" t="n"/>
+      <c r="G182" s="4" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="H182" s="6" t="n"/>
+      <c r="I182" s="6" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="J182" s="6" t="n">
         <v>41</v>
       </c>
-      <c r="K182" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K182" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
     <row r="183">
-      <c r="A183" s="2" t="inlineStr">
+      <c r="A183" s="4" t="inlineStr">
         <is>
           <t>5C</t>
         </is>
       </c>
-      <c r="B183" s="3" t="inlineStr">
+      <c r="B183" s="5" t="inlineStr">
         <is>
           <t>SL 72 RS</t>
         </is>
       </c>
-      <c r="C183" s="2" t="inlineStr">
+      <c r="C183" s="4" t="inlineStr">
         <is>
           <t>KJ1672</t>
         </is>
       </c>
-      <c r="D183" s="2" t="n">
+      <c r="D183" s="4" t="n">
         <v>2908</v>
       </c>
-      <c r="E183" s="2" t="n"/>
-      <c r="F183" s="2" t="n"/>
-      <c r="G183" s="2" t="n"/>
-      <c r="H183" s="2" t="n"/>
-      <c r="I183" s="2" t="n"/>
-      <c r="J183" s="2" t="n">
+      <c r="E183" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="F183" s="6" t="n"/>
+      <c r="G183" s="4" t="n">
+        <v>35.5</v>
+      </c>
+      <c r="H183" s="6" t="n"/>
+      <c r="I183" s="6" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="J183" s="6" t="n">
         <v>41</v>
       </c>
-      <c r="K183" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K183" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
     <row r="184">
-      <c r="A184" s="2" t="inlineStr">
+      <c r="A184" s="4" t="inlineStr">
         <is>
           <t>5C</t>
         </is>
       </c>
-      <c r="B184" s="3" t="inlineStr">
+      <c r="B184" s="5" t="inlineStr">
         <is>
           <t>SL 72 RS</t>
         </is>
       </c>
-      <c r="C184" s="2" t="inlineStr">
+      <c r="C184" s="4" t="inlineStr">
         <is>
           <t>KJ1673</t>
         </is>
       </c>
-      <c r="D184" s="2" t="n">
+      <c r="D184" s="4" t="n">
         <v>1140</v>
       </c>
-      <c r="E184" s="2" t="n"/>
-      <c r="F184" s="2" t="n"/>
-      <c r="G184" s="2" t="n"/>
-      <c r="H184" s="2" t="n"/>
-      <c r="I184" s="2" t="n"/>
-      <c r="J184" s="2" t="n">
+      <c r="E184" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="F184" s="6" t="n"/>
+      <c r="G184" s="4" t="n">
+        <v>35.5</v>
+      </c>
+      <c r="H184" s="6" t="n"/>
+      <c r="I184" s="6" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="J184" s="6" t="n">
         <v>41</v>
       </c>
-      <c r="K184" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K184" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
@@ -7906,76 +8164,88 @@
       </c>
     </row>
     <row r="189">
-      <c r="A189" s="2" t="inlineStr">
+      <c r="A189" s="4" t="inlineStr">
         <is>
           <t>6A</t>
         </is>
       </c>
-      <c r="B189" s="3" t="inlineStr">
+      <c r="B189" s="5" t="inlineStr">
         <is>
           <t>OZGAIA W</t>
         </is>
       </c>
-      <c r="C189" s="2" t="inlineStr">
+      <c r="C189" s="4" t="inlineStr">
         <is>
           <t>IG6047</t>
         </is>
       </c>
-      <c r="D189" s="2" t="n">
+      <c r="D189" s="4" t="n">
         <v>154</v>
       </c>
-      <c r="E189" s="2" t="n"/>
-      <c r="F189" s="2" t="n">
+      <c r="E189" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="F189" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="G189" s="2" t="n"/>
-      <c r="H189" s="2" t="n">
+      <c r="G189" s="4" t="n">
         <v>41</v>
       </c>
-      <c r="I189" s="2" t="n"/>
-      <c r="J189" s="2" t="n">
+      <c r="H189" s="4" t="n">
+        <v>41</v>
+      </c>
+      <c r="I189" s="4" t="n">
         <v>36</v>
       </c>
-      <c r="K189" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="J189" s="4" t="n">
+        <v>36</v>
+      </c>
+      <c r="K189" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
     <row r="190">
-      <c r="A190" s="2" t="inlineStr">
+      <c r="A190" s="4" t="inlineStr">
         <is>
           <t>6A</t>
         </is>
       </c>
-      <c r="B190" s="3" t="inlineStr">
+      <c r="B190" s="5" t="inlineStr">
         <is>
           <t>OZGAIA W</t>
         </is>
       </c>
-      <c r="C190" s="2" t="inlineStr">
+      <c r="C190" s="4" t="inlineStr">
         <is>
           <t>IG6049</t>
         </is>
       </c>
-      <c r="D190" s="2" t="n">
+      <c r="D190" s="4" t="n">
         <v>1007</v>
       </c>
-      <c r="E190" s="2" t="n"/>
-      <c r="F190" s="2" t="n">
+      <c r="E190" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="F190" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="G190" s="2" t="n"/>
-      <c r="H190" s="2" t="n">
+      <c r="G190" s="4" t="n">
         <v>41</v>
       </c>
-      <c r="I190" s="2" t="n"/>
-      <c r="J190" s="2" t="n">
+      <c r="H190" s="4" t="n">
+        <v>41</v>
+      </c>
+      <c r="I190" s="4" t="n">
         <v>36</v>
       </c>
-      <c r="K190" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="J190" s="4" t="n">
+        <v>36</v>
+      </c>
+      <c r="K190" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
@@ -8109,39 +8379,45 @@
       </c>
     </row>
     <row r="194">
-      <c r="A194" s="2" t="inlineStr">
+      <c r="A194" s="4" t="inlineStr">
         <is>
           <t>6A</t>
         </is>
       </c>
-      <c r="B194" s="3" t="inlineStr">
+      <c r="B194" s="5" t="inlineStr">
         <is>
           <t>OZGAIA W</t>
         </is>
       </c>
-      <c r="C194" s="2" t="inlineStr">
+      <c r="C194" s="4" t="inlineStr">
         <is>
           <t>KZ7072</t>
         </is>
       </c>
-      <c r="D194" s="2" t="n">
+      <c r="D194" s="4" t="n">
         <v>2734</v>
       </c>
-      <c r="E194" s="2" t="n"/>
-      <c r="F194" s="2" t="n">
+      <c r="E194" s="6" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="F194" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="G194" s="2" t="n"/>
-      <c r="H194" s="2" t="n">
+      <c r="G194" s="6" t="n">
+        <v>44</v>
+      </c>
+      <c r="H194" s="6" t="n">
         <v>41</v>
       </c>
-      <c r="I194" s="2" t="n"/>
-      <c r="J194" s="2" t="n">
+      <c r="I194" s="6" t="n">
+        <v>37</v>
+      </c>
+      <c r="J194" s="6" t="n">
         <v>36</v>
       </c>
-      <c r="K194" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K194" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
@@ -8361,76 +8637,88 @@
       </c>
     </row>
     <row r="200">
-      <c r="A200" s="2" t="inlineStr">
+      <c r="A200" s="4" t="inlineStr">
         <is>
           <t>6B</t>
         </is>
       </c>
-      <c r="B200" s="3" t="inlineStr">
+      <c r="B200" s="5" t="inlineStr">
         <is>
           <t>GHOST SPRINT W</t>
         </is>
       </c>
-      <c r="C200" s="2" t="inlineStr">
+      <c r="C200" s="4" t="inlineStr">
         <is>
           <t>KI4564</t>
         </is>
       </c>
-      <c r="D200" s="2" t="n">
+      <c r="D200" s="4" t="n">
         <v>201</v>
       </c>
-      <c r="E200" s="2" t="n"/>
-      <c r="F200" s="2" t="n">
+      <c r="E200" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="F200" s="6" t="n">
         <v>17</v>
       </c>
-      <c r="G200" s="2" t="n"/>
-      <c r="H200" s="2" t="n">
+      <c r="G200" s="4" t="n">
         <v>45</v>
       </c>
-      <c r="I200" s="2" t="n"/>
-      <c r="J200" s="2" t="n">
+      <c r="H200" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="I200" s="6" t="n">
+        <v>53</v>
+      </c>
+      <c r="J200" s="6" t="n">
         <v>61</v>
       </c>
-      <c r="K200" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K200" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
     <row r="201">
-      <c r="A201" s="2" t="inlineStr">
+      <c r="A201" s="4" t="inlineStr">
         <is>
           <t>6B</t>
         </is>
       </c>
-      <c r="B201" s="3" t="inlineStr">
+      <c r="B201" s="5" t="inlineStr">
         <is>
           <t>GHOST SPRINT W</t>
         </is>
       </c>
-      <c r="C201" s="2" t="inlineStr">
+      <c r="C201" s="4" t="inlineStr">
         <is>
           <t>KI4568</t>
         </is>
       </c>
-      <c r="D201" s="2" t="n">
+      <c r="D201" s="4" t="n">
         <v>694</v>
       </c>
-      <c r="E201" s="2" t="n"/>
-      <c r="F201" s="2" t="n">
+      <c r="E201" s="4" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="F201" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="G201" s="2" t="n"/>
-      <c r="H201" s="2" t="n">
+      <c r="G201" s="6" t="n">
+        <v>47</v>
+      </c>
+      <c r="H201" s="6" t="n">
         <v>45</v>
       </c>
-      <c r="I201" s="2" t="n"/>
-      <c r="J201" s="2" t="n">
+      <c r="I201" s="6" t="n">
+        <v>57</v>
+      </c>
+      <c r="J201" s="6" t="n">
         <v>61</v>
       </c>
-      <c r="K201" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K201" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
@@ -8478,39 +8766,45 @@
       </c>
     </row>
     <row r="203">
-      <c r="A203" s="2" t="inlineStr">
+      <c r="A203" s="4" t="inlineStr">
         <is>
           <t>6B</t>
         </is>
       </c>
-      <c r="B203" s="3" t="inlineStr">
+      <c r="B203" s="5" t="inlineStr">
         <is>
           <t>GHOST SPRINT W</t>
         </is>
       </c>
-      <c r="C203" s="2" t="inlineStr">
+      <c r="C203" s="4" t="inlineStr">
         <is>
           <t>KI4570</t>
         </is>
       </c>
-      <c r="D203" s="2" t="n">
+      <c r="D203" s="4" t="n">
         <v>50</v>
       </c>
-      <c r="E203" s="2" t="n"/>
-      <c r="F203" s="2" t="n">
+      <c r="E203" s="6" t="n">
+        <v>29.5</v>
+      </c>
+      <c r="F203" s="6" t="n">
         <v>17</v>
       </c>
-      <c r="G203" s="2" t="n"/>
-      <c r="H203" s="2" t="n">
+      <c r="G203" s="6" t="n">
+        <v>46</v>
+      </c>
+      <c r="H203" s="6" t="n">
         <v>45</v>
       </c>
-      <c r="I203" s="2" t="n"/>
-      <c r="J203" s="2" t="n">
+      <c r="I203" s="6" t="n">
+        <v>58</v>
+      </c>
+      <c r="J203" s="6" t="n">
         <v>61</v>
       </c>
-      <c r="K203" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K203" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
@@ -8558,39 +8852,45 @@
       </c>
     </row>
     <row r="205">
-      <c r="A205" s="2" t="inlineStr">
+      <c r="A205" s="4" t="inlineStr">
         <is>
           <t>6B</t>
         </is>
       </c>
-      <c r="B205" s="3" t="inlineStr">
+      <c r="B205" s="5" t="inlineStr">
         <is>
           <t>GHOST SPRINT W</t>
         </is>
       </c>
-      <c r="C205" s="2" t="inlineStr">
+      <c r="C205" s="4" t="inlineStr">
         <is>
           <t>KI4572</t>
         </is>
       </c>
-      <c r="D205" s="2" t="n">
+      <c r="D205" s="4" t="n">
         <v>70</v>
       </c>
-      <c r="E205" s="2" t="n"/>
-      <c r="F205" s="2" t="n">
+      <c r="E205" s="6" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="F205" s="6" t="n">
         <v>17</v>
       </c>
-      <c r="G205" s="2" t="n"/>
-      <c r="H205" s="2" t="n">
+      <c r="G205" s="6" t="n">
+        <v>46</v>
+      </c>
+      <c r="H205" s="6" t="n">
         <v>45</v>
       </c>
-      <c r="I205" s="2" t="n"/>
-      <c r="J205" s="2" t="n">
+      <c r="I205" s="4" t="n">
         <v>61</v>
       </c>
-      <c r="K205" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="J205" s="4" t="n">
+        <v>61</v>
+      </c>
+      <c r="K205" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
@@ -8638,76 +8938,88 @@
       </c>
     </row>
     <row r="207">
-      <c r="A207" s="2" t="inlineStr">
+      <c r="A207" s="4" t="inlineStr">
         <is>
           <t>6B</t>
         </is>
       </c>
-      <c r="B207" s="3" t="inlineStr">
+      <c r="B207" s="5" t="inlineStr">
         <is>
           <t>GHOST SPRINT W</t>
         </is>
       </c>
-      <c r="C207" s="2" t="inlineStr">
+      <c r="C207" s="4" t="inlineStr">
         <is>
           <t>KJ0645</t>
         </is>
       </c>
-      <c r="D207" s="2" t="n">
+      <c r="D207" s="4" t="n">
         <v>740</v>
       </c>
-      <c r="E207" s="2" t="n"/>
-      <c r="F207" s="2" t="n">
+      <c r="E207" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="F207" s="6" t="n">
         <v>17</v>
       </c>
-      <c r="G207" s="2" t="n"/>
-      <c r="H207" s="2" t="n">
+      <c r="G207" s="6" t="n">
+        <v>46</v>
+      </c>
+      <c r="H207" s="6" t="n">
         <v>45</v>
       </c>
-      <c r="I207" s="2" t="n"/>
-      <c r="J207" s="2" t="n">
+      <c r="I207" s="6" t="n">
+        <v>58</v>
+      </c>
+      <c r="J207" s="6" t="n">
         <v>61</v>
       </c>
-      <c r="K207" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K207" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
     <row r="208">
-      <c r="A208" s="2" t="inlineStr">
+      <c r="A208" s="4" t="inlineStr">
         <is>
           <t>6B</t>
         </is>
       </c>
-      <c r="B208" s="3" t="inlineStr">
+      <c r="B208" s="5" t="inlineStr">
         <is>
           <t>GHOST SPRINT W</t>
         </is>
       </c>
-      <c r="C208" s="2" t="inlineStr">
+      <c r="C208" s="4" t="inlineStr">
         <is>
           <t>KJ0646</t>
         </is>
       </c>
-      <c r="D208" s="2" t="n">
+      <c r="D208" s="4" t="n">
         <v>789</v>
       </c>
-      <c r="E208" s="2" t="n"/>
-      <c r="F208" s="2" t="n">
+      <c r="E208" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="F208" s="6" t="n">
         <v>17</v>
       </c>
-      <c r="G208" s="2" t="n"/>
-      <c r="H208" s="2" t="n">
+      <c r="G208" s="6" t="n">
+        <v>46</v>
+      </c>
+      <c r="H208" s="6" t="n">
         <v>45</v>
       </c>
-      <c r="I208" s="2" t="n"/>
-      <c r="J208" s="2" t="n">
+      <c r="I208" s="6" t="n">
+        <v>58</v>
+      </c>
+      <c r="J208" s="6" t="n">
         <v>61</v>
       </c>
-      <c r="K208" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K208" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
@@ -8946,19 +9258,19 @@
         <v>2329</v>
       </c>
       <c r="E214" s="6" t="n">
-        <v>10.5</v>
+        <v>19</v>
       </c>
       <c r="F214" s="6" t="n">
         <v>20</v>
       </c>
       <c r="G214" s="6" t="n">
-        <v>21</v>
+        <v>38</v>
       </c>
       <c r="H214" s="6" t="n">
         <v>37</v>
       </c>
       <c r="I214" s="6" t="n">
-        <v>20.5</v>
+        <v>35</v>
       </c>
       <c r="J214" s="6" t="n">
         <v>39</v>
@@ -9407,39 +9719,45 @@
       </c>
     </row>
     <row r="226">
-      <c r="A226" s="2" t="inlineStr">
+      <c r="A226" s="4" t="inlineStr">
         <is>
           <t>8B</t>
         </is>
       </c>
-      <c r="B226" s="3" t="inlineStr">
+      <c r="B226" s="5" t="inlineStr">
         <is>
           <t>GHOST SPRINT BALLET W</t>
         </is>
       </c>
-      <c r="C226" s="2" t="inlineStr">
+      <c r="C226" s="4" t="inlineStr">
         <is>
           <t>HQ7637</t>
         </is>
       </c>
-      <c r="D226" s="2" t="n">
+      <c r="D226" s="4" t="n">
         <v>182</v>
       </c>
-      <c r="E226" s="2" t="n"/>
-      <c r="F226" s="2" t="n">
+      <c r="E226" s="6" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="F226" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="G226" s="2" t="n"/>
-      <c r="H226" s="2" t="n">
+      <c r="G226" s="4" t="n">
         <v>38</v>
       </c>
-      <c r="I226" s="2" t="n"/>
-      <c r="J226" s="2" t="n">
+      <c r="H226" s="4" t="n">
+        <v>38</v>
+      </c>
+      <c r="I226" s="6" t="n">
+        <v>51.5</v>
+      </c>
+      <c r="J226" s="6" t="n">
         <v>45</v>
       </c>
-      <c r="K226" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K226" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
@@ -9604,76 +9922,88 @@
       </c>
     </row>
     <row r="231">
-      <c r="A231" s="2" t="inlineStr">
+      <c r="A231" s="4" t="inlineStr">
         <is>
           <t>8B</t>
         </is>
       </c>
-      <c r="B231" s="3" t="inlineStr">
+      <c r="B231" s="5" t="inlineStr">
         <is>
           <t>GHOST SPRINT BALLET W</t>
         </is>
       </c>
-      <c r="C231" s="2" t="inlineStr">
+      <c r="C231" s="4" t="inlineStr">
         <is>
           <t>KI7739</t>
         </is>
       </c>
-      <c r="D231" s="2" t="n">
+      <c r="D231" s="4" t="n">
         <v>426</v>
       </c>
-      <c r="E231" s="2" t="n"/>
-      <c r="F231" s="2" t="n">
+      <c r="E231" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="G231" s="2" t="n"/>
-      <c r="H231" s="2" t="n">
+      <c r="F231" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="G231" s="4" t="n">
         <v>38</v>
       </c>
-      <c r="I231" s="2" t="n"/>
-      <c r="J231" s="2" t="n">
+      <c r="H231" s="4" t="n">
+        <v>38</v>
+      </c>
+      <c r="I231" s="4" t="n">
+        <v>44.5</v>
+      </c>
+      <c r="J231" s="4" t="n">
         <v>45</v>
       </c>
-      <c r="K231" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K231" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
     <row r="232">
-      <c r="A232" s="2" t="inlineStr">
+      <c r="A232" s="4" t="inlineStr">
         <is>
           <t>8B</t>
         </is>
       </c>
-      <c r="B232" s="3" t="inlineStr">
+      <c r="B232" s="5" t="inlineStr">
         <is>
           <t>GHOST SPRINT BALLET W</t>
         </is>
       </c>
-      <c r="C232" s="2" t="inlineStr">
+      <c r="C232" s="4" t="inlineStr">
         <is>
           <t>KI7740</t>
         </is>
       </c>
-      <c r="D232" s="2" t="n">
+      <c r="D232" s="4" t="n">
         <v>1471</v>
       </c>
-      <c r="E232" s="2" t="n"/>
-      <c r="F232" s="2" t="n">
+      <c r="E232" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="G232" s="2" t="n"/>
-      <c r="H232" s="2" t="n">
+      <c r="F232" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="G232" s="4" t="n">
         <v>38</v>
       </c>
-      <c r="I232" s="2" t="n"/>
-      <c r="J232" s="2" t="n">
+      <c r="H232" s="4" t="n">
+        <v>38</v>
+      </c>
+      <c r="I232" s="4" t="n">
+        <v>44.5</v>
+      </c>
+      <c r="J232" s="4" t="n">
         <v>45</v>
       </c>
-      <c r="K232" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K232" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
@@ -9752,39 +10082,45 @@
       </c>
     </row>
     <row r="235">
-      <c r="A235" s="2" t="inlineStr">
+      <c r="A235" s="4" t="inlineStr">
         <is>
           <t>8B</t>
         </is>
       </c>
-      <c r="B235" s="3" t="inlineStr">
+      <c r="B235" s="5" t="inlineStr">
         <is>
           <t>GHOST SPRINT BALLET W</t>
         </is>
       </c>
-      <c r="C235" s="2" t="inlineStr">
+      <c r="C235" s="4" t="inlineStr">
         <is>
           <t>KZ7291</t>
         </is>
       </c>
-      <c r="D235" s="2" t="n">
+      <c r="D235" s="4" t="n">
         <v>615</v>
       </c>
-      <c r="E235" s="2" t="n"/>
-      <c r="F235" s="2" t="n">
+      <c r="E235" s="4" t="n">
         <v>20</v>
       </c>
-      <c r="G235" s="2" t="n"/>
-      <c r="H235" s="2" t="n">
+      <c r="F235" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="G235" s="4" t="n">
         <v>38</v>
       </c>
-      <c r="I235" s="2" t="n"/>
-      <c r="J235" s="2" t="n">
+      <c r="H235" s="4" t="n">
+        <v>38</v>
+      </c>
+      <c r="I235" s="4" t="n">
+        <v>44.5</v>
+      </c>
+      <c r="J235" s="4" t="n">
         <v>45</v>
       </c>
-      <c r="K235" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K235" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
@@ -11484,39 +11820,45 @@
       </c>
     </row>
     <row r="277">
-      <c r="A277" s="2" t="inlineStr">
+      <c r="A277" s="4" t="inlineStr">
         <is>
           <t>10C</t>
         </is>
       </c>
-      <c r="B277" s="3" t="inlineStr">
+      <c r="B277" s="5" t="inlineStr">
         <is>
           <t>TAEKWONDO MEI ELITE W</t>
         </is>
       </c>
-      <c r="C277" s="2" t="inlineStr">
+      <c r="C277" s="4" t="inlineStr">
         <is>
           <t>KK2576</t>
         </is>
       </c>
-      <c r="D277" s="2" t="n">
+      <c r="D277" s="4" t="n">
         <v>813</v>
       </c>
-      <c r="E277" s="2" t="n"/>
-      <c r="F277" s="2" t="n">
+      <c r="E277" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="G277" s="2" t="n"/>
-      <c r="H277" s="2" t="n">
+      <c r="F277" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="G277" s="4" t="n">
         <v>26</v>
       </c>
-      <c r="I277" s="2" t="n"/>
-      <c r="J277" s="2" t="n">
+      <c r="H277" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="I277" s="4" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="J277" s="4" t="n">
         <v>24</v>
       </c>
-      <c r="K277" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K277" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
@@ -12093,35 +12435,41 @@
       </c>
     </row>
     <row r="292">
-      <c r="A292" s="2" t="inlineStr">
+      <c r="A292" s="4" t="inlineStr">
         <is>
           <t>10C</t>
         </is>
       </c>
-      <c r="B292" s="3" t="inlineStr">
+      <c r="B292" s="5" t="inlineStr">
         <is>
           <t>HANDBALL SPEZIAL</t>
         </is>
       </c>
-      <c r="C292" s="2" t="inlineStr">
+      <c r="C292" s="4" t="inlineStr">
         <is>
           <t>KK3019</t>
         </is>
       </c>
-      <c r="D292" s="2" t="n">
+      <c r="D292" s="4" t="n">
         <v>1386</v>
       </c>
-      <c r="E292" s="2" t="n"/>
-      <c r="F292" s="2" t="n"/>
-      <c r="G292" s="2" t="n"/>
-      <c r="H292" s="2" t="n"/>
-      <c r="I292" s="2" t="n"/>
-      <c r="J292" s="2" t="n">
+      <c r="E292" s="4" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="F292" s="6" t="n"/>
+      <c r="G292" s="4" t="n">
+        <v>36</v>
+      </c>
+      <c r="H292" s="6" t="n"/>
+      <c r="I292" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="J292" s="6" t="n">
         <v>34</v>
       </c>
-      <c r="K292" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K292" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
@@ -12204,101 +12552,119 @@
       </c>
     </row>
     <row r="295">
-      <c r="A295" s="2" t="inlineStr">
+      <c r="A295" s="4" t="inlineStr">
         <is>
           <t>10C</t>
         </is>
       </c>
-      <c r="B295" s="3" t="inlineStr">
+      <c r="B295" s="5" t="inlineStr">
         <is>
           <t>HANDBALL SPEZIAL</t>
         </is>
       </c>
-      <c r="C295" s="2" t="inlineStr">
+      <c r="C295" s="4" t="inlineStr">
         <is>
           <t>KK3026</t>
         </is>
       </c>
-      <c r="D295" s="2" t="n">
+      <c r="D295" s="4" t="n">
         <v>216</v>
       </c>
-      <c r="E295" s="2" t="n"/>
-      <c r="F295" s="2" t="n"/>
-      <c r="G295" s="2" t="n"/>
-      <c r="H295" s="2" t="n"/>
-      <c r="I295" s="2" t="n"/>
-      <c r="J295" s="2" t="n">
+      <c r="E295" s="4" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="F295" s="6" t="n"/>
+      <c r="G295" s="4" t="n">
+        <v>36</v>
+      </c>
+      <c r="H295" s="6" t="n"/>
+      <c r="I295" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="J295" s="6" t="n">
         <v>34</v>
       </c>
-      <c r="K295" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K295" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
     <row r="296">
-      <c r="A296" s="2" t="inlineStr">
+      <c r="A296" s="4" t="inlineStr">
         <is>
           <t>10C</t>
         </is>
       </c>
-      <c r="B296" s="3" t="inlineStr">
+      <c r="B296" s="5" t="inlineStr">
         <is>
           <t>HANDBALL SPEZIAL</t>
         </is>
       </c>
-      <c r="C296" s="2" t="inlineStr">
+      <c r="C296" s="4" t="inlineStr">
         <is>
           <t>KK3027</t>
         </is>
       </c>
-      <c r="D296" s="2" t="n">
+      <c r="D296" s="4" t="n">
         <v>216</v>
       </c>
-      <c r="E296" s="2" t="n"/>
-      <c r="F296" s="2" t="n"/>
-      <c r="G296" s="2" t="n"/>
-      <c r="H296" s="2" t="n"/>
-      <c r="I296" s="2" t="n"/>
-      <c r="J296" s="2" t="n">
+      <c r="E296" s="4" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="F296" s="6" t="n"/>
+      <c r="G296" s="4" t="n">
+        <v>36</v>
+      </c>
+      <c r="H296" s="6" t="n"/>
+      <c r="I296" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="J296" s="6" t="n">
         <v>34</v>
       </c>
-      <c r="K296" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K296" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
     <row r="297">
-      <c r="A297" s="2" t="inlineStr">
+      <c r="A297" s="4" t="inlineStr">
         <is>
           <t>10C</t>
         </is>
       </c>
-      <c r="B297" s="3" t="inlineStr">
+      <c r="B297" s="5" t="inlineStr">
         <is>
           <t>HANDBALL SPEZIAL</t>
         </is>
       </c>
-      <c r="C297" s="2" t="inlineStr">
+      <c r="C297" s="4" t="inlineStr">
         <is>
           <t>KK3033</t>
         </is>
       </c>
-      <c r="D297" s="2" t="n">
+      <c r="D297" s="4" t="n">
         <v>192</v>
       </c>
-      <c r="E297" s="2" t="n"/>
-      <c r="F297" s="2" t="n"/>
-      <c r="G297" s="2" t="n"/>
-      <c r="H297" s="2" t="n"/>
-      <c r="I297" s="2" t="n"/>
-      <c r="J297" s="2" t="n">
+      <c r="E297" s="4" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="F297" s="6" t="n"/>
+      <c r="G297" s="4" t="n">
+        <v>36</v>
+      </c>
+      <c r="H297" s="6" t="n"/>
+      <c r="I297" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="J297" s="6" t="n">
         <v>34</v>
       </c>
-      <c r="K297" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K297" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
@@ -12342,200 +12708,236 @@
       </c>
     </row>
     <row r="299">
-      <c r="A299" s="2" t="inlineStr">
+      <c r="A299" s="4" t="inlineStr">
         <is>
           <t>12A</t>
         </is>
       </c>
-      <c r="B299" s="3" t="inlineStr">
+      <c r="B299" s="5" t="inlineStr">
         <is>
           <t>1609ER RS</t>
         </is>
       </c>
-      <c r="C299" s="2" t="inlineStr">
+      <c r="C299" s="4" t="inlineStr">
         <is>
           <t>HQ5207</t>
         </is>
       </c>
-      <c r="D299" s="2" t="n">
+      <c r="D299" s="4" t="n">
         <v>2960</v>
       </c>
-      <c r="E299" s="2" t="n"/>
-      <c r="F299" s="2" t="n"/>
-      <c r="G299" s="2" t="n"/>
-      <c r="H299" s="2" t="n"/>
-      <c r="I299" s="2" t="n"/>
-      <c r="J299" s="2" t="n">
+      <c r="E299" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="F299" s="6" t="n"/>
+      <c r="G299" s="4" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="H299" s="6" t="n"/>
+      <c r="I299" s="6" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="J299" s="6" t="n">
         <v>24</v>
       </c>
-      <c r="K299" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K299" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
     <row r="300">
-      <c r="A300" s="2" t="inlineStr">
+      <c r="A300" s="4" t="inlineStr">
         <is>
           <t>12A</t>
         </is>
       </c>
-      <c r="B300" s="3" t="inlineStr">
+      <c r="B300" s="5" t="inlineStr">
         <is>
           <t>1609ER RS</t>
         </is>
       </c>
-      <c r="C300" s="2" t="inlineStr">
+      <c r="C300" s="4" t="inlineStr">
         <is>
           <t>HQ5208</t>
         </is>
       </c>
-      <c r="D300" s="2" t="n">
+      <c r="D300" s="4" t="n">
         <v>1629</v>
       </c>
-      <c r="E300" s="2" t="n"/>
-      <c r="F300" s="2" t="n"/>
-      <c r="G300" s="2" t="n"/>
-      <c r="H300" s="2" t="n"/>
-      <c r="I300" s="2" t="n"/>
-      <c r="J300" s="2" t="n">
+      <c r="E300" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="F300" s="6" t="n"/>
+      <c r="G300" s="4" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="H300" s="6" t="n"/>
+      <c r="I300" s="6" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="J300" s="6" t="n">
         <v>24</v>
       </c>
-      <c r="K300" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K300" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
     <row r="301">
-      <c r="A301" s="2" t="inlineStr">
+      <c r="A301" s="4" t="inlineStr">
         <is>
           <t>12A</t>
         </is>
       </c>
-      <c r="B301" s="3" t="inlineStr">
+      <c r="B301" s="5" t="inlineStr">
         <is>
           <t>1609ER RS</t>
         </is>
       </c>
-      <c r="C301" s="2" t="inlineStr">
+      <c r="C301" s="4" t="inlineStr">
         <is>
           <t>HQ5209</t>
         </is>
       </c>
-      <c r="D301" s="2" t="n">
+      <c r="D301" s="4" t="n">
         <v>2229</v>
       </c>
-      <c r="E301" s="2" t="n"/>
-      <c r="F301" s="2" t="n"/>
-      <c r="G301" s="2" t="n"/>
-      <c r="H301" s="2" t="n"/>
-      <c r="I301" s="2" t="n"/>
-      <c r="J301" s="2" t="n">
+      <c r="E301" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="F301" s="6" t="n"/>
+      <c r="G301" s="4" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="H301" s="6" t="n"/>
+      <c r="I301" s="6" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="J301" s="6" t="n">
         <v>24</v>
       </c>
-      <c r="K301" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K301" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
     <row r="302">
-      <c r="A302" s="2" t="inlineStr">
+      <c r="A302" s="4" t="inlineStr">
         <is>
           <t>12A</t>
         </is>
       </c>
-      <c r="B302" s="3" t="inlineStr">
+      <c r="B302" s="5" t="inlineStr">
         <is>
           <t>1609ER RS</t>
         </is>
       </c>
-      <c r="C302" s="2" t="inlineStr">
+      <c r="C302" s="4" t="inlineStr">
         <is>
           <t>KH9907</t>
         </is>
       </c>
-      <c r="D302" s="2" t="n">
+      <c r="D302" s="4" t="n">
         <v>2589</v>
       </c>
-      <c r="E302" s="2" t="n"/>
-      <c r="F302" s="2" t="n"/>
-      <c r="G302" s="2" t="n"/>
-      <c r="H302" s="2" t="n"/>
-      <c r="I302" s="2" t="n"/>
-      <c r="J302" s="2" t="n">
+      <c r="E302" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="F302" s="6" t="n"/>
+      <c r="G302" s="4" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="H302" s="6" t="n"/>
+      <c r="I302" s="6" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="J302" s="6" t="n">
         <v>24</v>
       </c>
-      <c r="K302" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K302" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
     <row r="303">
-      <c r="A303" s="2" t="inlineStr">
+      <c r="A303" s="4" t="inlineStr">
         <is>
           <t>12A</t>
         </is>
       </c>
-      <c r="B303" s="3" t="inlineStr">
+      <c r="B303" s="5" t="inlineStr">
         <is>
           <t>1609ER RS</t>
         </is>
       </c>
-      <c r="C303" s="2" t="inlineStr">
+      <c r="C303" s="4" t="inlineStr">
         <is>
           <t>KH9908</t>
         </is>
       </c>
-      <c r="D303" s="2" t="n">
+      <c r="D303" s="4" t="n">
         <v>554</v>
       </c>
-      <c r="E303" s="2" t="n"/>
-      <c r="F303" s="2" t="n"/>
-      <c r="G303" s="2" t="n"/>
-      <c r="H303" s="2" t="n"/>
-      <c r="I303" s="2" t="n"/>
-      <c r="J303" s="2" t="n">
+      <c r="E303" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="F303" s="6" t="n"/>
+      <c r="G303" s="4" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="H303" s="6" t="n"/>
+      <c r="I303" s="6" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="J303" s="6" t="n">
         <v>24</v>
       </c>
-      <c r="K303" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K303" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
     <row r="304">
-      <c r="A304" s="2" t="inlineStr">
+      <c r="A304" s="4" t="inlineStr">
         <is>
           <t>12A</t>
         </is>
       </c>
-      <c r="B304" s="3" t="inlineStr">
+      <c r="B304" s="5" t="inlineStr">
         <is>
           <t>1609ER RS</t>
         </is>
       </c>
-      <c r="C304" s="2" t="inlineStr">
+      <c r="C304" s="4" t="inlineStr">
         <is>
           <t>KH9909</t>
         </is>
       </c>
-      <c r="D304" s="2" t="n">
+      <c r="D304" s="4" t="n">
         <v>107</v>
       </c>
-      <c r="E304" s="2" t="n"/>
-      <c r="F304" s="2" t="n"/>
-      <c r="G304" s="2" t="n"/>
-      <c r="H304" s="2" t="n"/>
-      <c r="I304" s="2" t="n"/>
-      <c r="J304" s="2" t="n">
+      <c r="E304" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="F304" s="6" t="n"/>
+      <c r="G304" s="4" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="H304" s="6" t="n"/>
+      <c r="I304" s="6" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="J304" s="6" t="n">
         <v>24</v>
       </c>
-      <c r="K304" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K304" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
@@ -12579,68 +12981,80 @@
       </c>
     </row>
     <row r="306">
-      <c r="A306" s="2" t="inlineStr">
+      <c r="A306" s="4" t="inlineStr">
         <is>
           <t>12A</t>
         </is>
       </c>
-      <c r="B306" s="3" t="inlineStr">
+      <c r="B306" s="5" t="inlineStr">
         <is>
           <t>1609ER RS</t>
         </is>
       </c>
-      <c r="C306" s="2" t="inlineStr">
+      <c r="C306" s="4" t="inlineStr">
         <is>
           <t>KI9855</t>
         </is>
       </c>
-      <c r="D306" s="2" t="n">
+      <c r="D306" s="4" t="n">
         <v>442</v>
       </c>
-      <c r="E306" s="2" t="n"/>
-      <c r="F306" s="2" t="n"/>
-      <c r="G306" s="2" t="n"/>
-      <c r="H306" s="2" t="n"/>
-      <c r="I306" s="2" t="n"/>
-      <c r="J306" s="2" t="n">
+      <c r="E306" s="4" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="F306" s="6" t="n"/>
+      <c r="G306" s="4" t="n">
+        <v>33.5</v>
+      </c>
+      <c r="H306" s="6" t="n"/>
+      <c r="I306" s="6" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="J306" s="6" t="n">
         <v>24</v>
       </c>
-      <c r="K306" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K306" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
     <row r="307">
-      <c r="A307" s="2" t="inlineStr">
+      <c r="A307" s="4" t="inlineStr">
         <is>
           <t>12A</t>
         </is>
       </c>
-      <c r="B307" s="3" t="inlineStr">
+      <c r="B307" s="5" t="inlineStr">
         <is>
           <t>1609ER RS</t>
         </is>
       </c>
-      <c r="C307" s="2" t="inlineStr">
+      <c r="C307" s="4" t="inlineStr">
         <is>
           <t>KI9857</t>
         </is>
       </c>
-      <c r="D307" s="2" t="n">
+      <c r="D307" s="4" t="n">
         <v>395</v>
       </c>
-      <c r="E307" s="2" t="n"/>
-      <c r="F307" s="2" t="n"/>
-      <c r="G307" s="2" t="n"/>
-      <c r="H307" s="2" t="n"/>
-      <c r="I307" s="2" t="n"/>
-      <c r="J307" s="2" t="n">
+      <c r="E307" s="4" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="F307" s="6" t="n"/>
+      <c r="G307" s="4" t="n">
+        <v>33.5</v>
+      </c>
+      <c r="H307" s="6" t="n"/>
+      <c r="I307" s="6" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="J307" s="6" t="n">
         <v>24</v>
       </c>
-      <c r="K307" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K307" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
@@ -12678,35 +13092,41 @@
       </c>
     </row>
     <row r="309">
-      <c r="A309" s="2" t="inlineStr">
+      <c r="A309" s="4" t="inlineStr">
         <is>
           <t>12A</t>
         </is>
       </c>
-      <c r="B309" s="3" t="inlineStr">
+      <c r="B309" s="5" t="inlineStr">
         <is>
           <t>1609ER RS</t>
         </is>
       </c>
-      <c r="C309" s="2" t="inlineStr">
+      <c r="C309" s="4" t="inlineStr">
         <is>
           <t>KI9861</t>
         </is>
       </c>
-      <c r="D309" s="2" t="n">
+      <c r="D309" s="4" t="n">
         <v>172</v>
       </c>
-      <c r="E309" s="2" t="n"/>
-      <c r="F309" s="2" t="n"/>
-      <c r="G309" s="2" t="n"/>
-      <c r="H309" s="2" t="n"/>
-      <c r="I309" s="2" t="n"/>
-      <c r="J309" s="2" t="n">
+      <c r="E309" s="4" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="F309" s="6" t="n"/>
+      <c r="G309" s="4" t="n">
+        <v>33.5</v>
+      </c>
+      <c r="H309" s="6" t="n"/>
+      <c r="I309" s="6" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="J309" s="6" t="n">
         <v>24</v>
       </c>
-      <c r="K309" s="2" t="inlineStr">
-        <is>
-          <t>MISSING_IE</t>
+      <c r="K309" s="6" t="inlineStr">
+        <is>
+          <t>MISMATCH</t>
         </is>
       </c>
     </row>
@@ -12791,7 +13211,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>172</v>
+        <v>242</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -12806,7 +13226,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>137</v>
+        <v>67</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
2026-06-09 ie_sheet_data 導入 + 22 sheet tabs 動態顯示
</commit_message>
<xml_diff>
--- a/flask_backend/test_output/comparison_table.xlsx
+++ b/flask_backend/test_output/comparison_table.xlsx
@@ -833,21 +833,21 @@
         <v>2582</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="F9" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="G9" s="6" t="n">
-        <v>34.5</v>
-      </c>
-      <c r="H9" s="6" t="n">
+      <c r="G9" s="4" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="H9" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="I9" s="6" t="n">
-        <v>39</v>
-      </c>
-      <c r="J9" s="6" t="n">
+      <c r="I9" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="J9" s="4" t="n">
         <v>21</v>
       </c>
       <c r="K9" s="6" t="inlineStr">
@@ -876,21 +876,21 @@
         <v>800</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="F10" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="G10" s="6" t="n">
-        <v>34.5</v>
-      </c>
-      <c r="H10" s="6" t="n">
+      <c r="G10" s="4" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="H10" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="I10" s="6" t="n">
-        <v>39</v>
-      </c>
-      <c r="J10" s="6" t="n">
+      <c r="I10" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="J10" s="4" t="n">
         <v>21</v>
       </c>
       <c r="K10" s="6" t="inlineStr">
@@ -1306,21 +1306,21 @@
         <v>489</v>
       </c>
       <c r="E20" s="6" t="n">
-        <v>14.5</v>
+        <v>8.5</v>
       </c>
       <c r="F20" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="G20" s="6" t="n">
-        <v>30</v>
-      </c>
-      <c r="H20" s="6" t="n">
+      <c r="G20" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="I20" s="6" t="n">
-        <v>38</v>
-      </c>
-      <c r="J20" s="6" t="n">
+      <c r="H20" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="I20" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="J20" s="4" t="n">
         <v>21</v>
       </c>
       <c r="K20" s="6" t="inlineStr">
@@ -1349,21 +1349,21 @@
         <v>110</v>
       </c>
       <c r="E21" s="6" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="F21" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="G21" s="6" t="n">
-        <v>34.5</v>
-      </c>
-      <c r="H21" s="6" t="n">
+      <c r="G21" s="4" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="H21" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="I21" s="6" t="n">
-        <v>39</v>
-      </c>
-      <c r="J21" s="6" t="n">
+      <c r="I21" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="J21" s="4" t="n">
         <v>21</v>
       </c>
       <c r="K21" s="6" t="inlineStr">
@@ -3076,19 +3076,19 @@
         <v>598</v>
       </c>
       <c r="E62" s="6" t="n">
-        <v>6.5</v>
+        <v>13</v>
       </c>
       <c r="F62" s="6" t="n">
         <v>20</v>
       </c>
       <c r="G62" s="6" t="n">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="H62" s="6" t="n">
         <v>31</v>
       </c>
       <c r="I62" s="6" t="n">
-        <v>21.5</v>
+        <v>39.5</v>
       </c>
       <c r="J62" s="6" t="n">
         <v>41</v>
@@ -3118,20 +3118,20 @@
       <c r="D63" s="4" t="n">
         <v>221</v>
       </c>
-      <c r="E63" s="4" t="n">
-        <v>20.5</v>
-      </c>
-      <c r="F63" s="4" t="n">
+      <c r="E63" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="F63" s="6" t="n">
         <v>20</v>
       </c>
       <c r="G63" s="6" t="n">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="H63" s="6" t="n">
         <v>31</v>
       </c>
       <c r="I63" s="6" t="n">
-        <v>36.5</v>
+        <v>20.5</v>
       </c>
       <c r="J63" s="6" t="n">
         <v>41</v>
@@ -3462,20 +3462,20 @@
       <c r="D71" s="4" t="n">
         <v>637</v>
       </c>
-      <c r="E71" s="4" t="n">
-        <v>20.5</v>
-      </c>
-      <c r="F71" s="4" t="n">
+      <c r="E71" s="6" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="F71" s="6" t="n">
         <v>20</v>
       </c>
       <c r="G71" s="6" t="n">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="H71" s="6" t="n">
         <v>31</v>
       </c>
       <c r="I71" s="6" t="n">
-        <v>36.5</v>
+        <v>20.5</v>
       </c>
       <c r="J71" s="6" t="n">
         <v>41</v>
@@ -3763,20 +3763,20 @@
       <c r="D78" s="4" t="n">
         <v>240</v>
       </c>
-      <c r="E78" s="4" t="n">
+      <c r="E78" s="6" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="F78" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="F78" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="G78" s="4" t="n">
-        <v>31.5</v>
-      </c>
-      <c r="H78" s="4" t="n">
+      <c r="G78" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="H78" s="6" t="n">
         <v>31</v>
       </c>
       <c r="I78" s="6" t="n">
-        <v>43.5</v>
+        <v>23.5</v>
       </c>
       <c r="J78" s="6" t="n">
         <v>41</v>
@@ -3893,21 +3893,21 @@
         <v>487</v>
       </c>
       <c r="E81" s="6" t="n">
-        <v>10.5</v>
+        <v>21.5</v>
       </c>
       <c r="F81" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="G81" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="H81" s="6" t="n">
+      <c r="G81" s="4" t="n">
         <v>31</v>
       </c>
-      <c r="I81" s="6" t="n">
-        <v>22</v>
-      </c>
-      <c r="J81" s="6" t="n">
+      <c r="H81" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="I81" s="4" t="n">
+        <v>40.5</v>
+      </c>
+      <c r="J81" s="4" t="n">
         <v>41</v>
       </c>
       <c r="K81" s="6" t="inlineStr">
@@ -3979,19 +3979,19 @@
         <v>346</v>
       </c>
       <c r="E83" s="6" t="n">
-        <v>11.5</v>
+        <v>6</v>
       </c>
       <c r="F83" s="6" t="n">
         <v>20</v>
       </c>
       <c r="G83" s="6" t="n">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="H83" s="6" t="n">
         <v>31</v>
       </c>
       <c r="I83" s="6" t="n">
-        <v>38.5</v>
+        <v>21</v>
       </c>
       <c r="J83" s="6" t="n">
         <v>41</v>
@@ -4065,19 +4065,19 @@
         <v>1638</v>
       </c>
       <c r="E85" s="6" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="F85" s="6" t="n">
         <v>20</v>
       </c>
       <c r="G85" s="6" t="n">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="H85" s="6" t="n">
         <v>31</v>
       </c>
       <c r="I85" s="6" t="n">
-        <v>36.5</v>
+        <v>21</v>
       </c>
       <c r="J85" s="6" t="n">
         <v>41</v>
@@ -5689,19 +5689,19 @@
         <v>1336</v>
       </c>
       <c r="E125" s="6" t="n">
-        <v>16</v>
+        <v>15.5</v>
       </c>
       <c r="F125" s="6" t="n">
         <v>12</v>
       </c>
       <c r="G125" s="6" t="n">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="H125" s="6" t="n">
         <v>31</v>
       </c>
       <c r="I125" s="6" t="n">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="J125" s="6" t="n">
         <v>39</v>
@@ -5775,19 +5775,19 @@
         <v>2500</v>
       </c>
       <c r="E127" s="6" t="n">
-        <v>8.5</v>
+        <v>14.5</v>
       </c>
       <c r="F127" s="6" t="n">
         <v>12</v>
       </c>
       <c r="G127" s="6" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="H127" s="6" t="n">
         <v>31</v>
       </c>
       <c r="I127" s="6" t="n">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="J127" s="6" t="n">
         <v>39</v>
@@ -9258,19 +9258,19 @@
         <v>2329</v>
       </c>
       <c r="E214" s="6" t="n">
-        <v>19</v>
+        <v>10.5</v>
       </c>
       <c r="F214" s="6" t="n">
         <v>20</v>
       </c>
       <c r="G214" s="6" t="n">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="H214" s="6" t="n">
         <v>37</v>
       </c>
       <c r="I214" s="6" t="n">
-        <v>35</v>
+        <v>20.5</v>
       </c>
       <c r="J214" s="6" t="n">
         <v>39</v>
@@ -13000,15 +13000,15 @@
         <v>442</v>
       </c>
       <c r="E306" s="4" t="n">
-        <v>12.5</v>
+        <v>7</v>
       </c>
       <c r="F306" s="6" t="n"/>
       <c r="G306" s="4" t="n">
-        <v>33.5</v>
+        <v>17.5</v>
       </c>
       <c r="H306" s="6" t="n"/>
       <c r="I306" s="6" t="n">
-        <v>38.5</v>
+        <v>21.5</v>
       </c>
       <c r="J306" s="6" t="n">
         <v>24</v>
@@ -13039,15 +13039,15 @@
         <v>395</v>
       </c>
       <c r="E307" s="4" t="n">
-        <v>12.5</v>
+        <v>7</v>
       </c>
       <c r="F307" s="6" t="n"/>
       <c r="G307" s="4" t="n">
-        <v>33.5</v>
+        <v>17.5</v>
       </c>
       <c r="H307" s="6" t="n"/>
       <c r="I307" s="6" t="n">
-        <v>38.5</v>
+        <v>21.5</v>
       </c>
       <c r="J307" s="6" t="n">
         <v>24</v>
@@ -13111,15 +13111,15 @@
         <v>172</v>
       </c>
       <c r="E309" s="4" t="n">
-        <v>12.5</v>
+        <v>7</v>
       </c>
       <c r="F309" s="6" t="n"/>
       <c r="G309" s="4" t="n">
-        <v>33.5</v>
+        <v>17.5</v>
       </c>
       <c r="H309" s="6" t="n"/>
       <c r="I309" s="6" t="n">
-        <v>38.5</v>
+        <v>21.5</v>
       </c>
       <c r="J309" s="6" t="n">
         <v>24</v>

</xml_diff>